<commit_message>
Update the data to the workbook of 2026-09-01
873 sources, 10 markets, 37 trends, 33 platforms, 30 genres.

Copied from public/downloads/ by scripts/build-mirror.mjs in the site
repository. Every count in the README is read from data/downloads.json rather
than typed, so it describes the files beside it.
</commit_message>
<xml_diff>
--- a/games-research-starter-pack.xlsx
+++ b/games-research-starter-pack.xlsx
@@ -474,7 +474,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Compiled from the research workbook of 2026-08-28. https://games.thisisdelightful.com</t>
+          <t>Compiled from the research workbook of 2026-09-01. https://games.thisisdelightful.com</t>
         </is>
       </c>
     </row>
@@ -55231,7 +55231,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Analyst Matthew Ball's annual reports argue gaming's decade of growth engines is exhausted: revenue and cultural weight are at record highs, yet growth is elusive and player counts are retreating across much of the developed world, so revenue gains come from monetizing existing players harder rather than adding new ones.</t>
+          <t>Analyst Matthew Ball's annual reports argue gaming's decade of growth engines is exhausted: revenue and cultural weight are at record highs, yet growth is elusive and player counts are retreating across much of the developed world, so revenue gains come from monetizing existing players harder rather than adding new ones. The revenue half of that picture has since softened in the largest market: Circana put US spending down 10% year-on-year in July 2026 at $4.5bn, with hardware down 29% and new physical software at an all-time July low, even as average hardware selling prices rose 16%.</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -55246,7 +55246,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Jul 2026</t>
+          <t>Sep 2026</t>
         </is>
       </c>
     </row>
@@ -55273,7 +55273,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>GTA 6 launched at $80, settling speculation about $100 base games. Only Mario Kart World, GTA 6, and Elden Ring on Switch 2 have cleared $70 — Microsoft tried and retreated to $70 after backlash. Meanwhile a RAM-driven hardware crunch pushed consoles past $600 and GPUs, monitors, and memory sharply higher.</t>
+          <t>GTA 6 launched at $80, settling speculation about $100 base games. Only Mario Kart World, GTA 6, and Elden Ring on Switch 2 have cleared $70 — Microsoft tried and retreated to $70 after backlash. Meanwhile a RAM-driven hardware crunch pushed consoles past $600 and GPUs, monitors, and memory sharply higher. Nintendo raised Switch 2 to $500 in the US, Canada and Europe from 1 September 2026 (Japan from 25 May), citing memory and component costs, and said the new price still does not cover build cost; it put the hardware-cost impact on FY2027 earnings at about ¥100bn.</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -55288,7 +55288,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Jul 2026</t>
+          <t>Sep 2026</t>
         </is>
       </c>
     </row>
@@ -56464,7 +56464,7 @@
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>46235</t>
+          <t>Aug 2026</t>
         </is>
       </c>
     </row>
@@ -56506,7 +56506,7 @@
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>46235</t>
+          <t>Aug 2026</t>
         </is>
       </c>
     </row>
@@ -56548,7 +56548,7 @@
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>46235</t>
+          <t>Aug 2026</t>
         </is>
       </c>
     </row>
@@ -56590,7 +56590,7 @@
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>46235</t>
+          <t>Aug 2026</t>
         </is>
       </c>
     </row>
@@ -56632,7 +56632,7 @@
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>46235</t>
+          <t>Aug 2026</t>
         </is>
       </c>
     </row>
@@ -56674,7 +56674,7 @@
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>46235</t>
+          <t>Aug 2026</t>
         </is>
       </c>
     </row>
@@ -56716,7 +56716,7 @@
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>46235</t>
+          <t>Aug 2026</t>
         </is>
       </c>
     </row>
@@ -56965,18 +56965,18 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>The affordability crisis has migrated from software to silicon</t>
+          <t>How a surge in memory prices will affect the games industry</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Community</t>
+          <t>Reporting</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr"/>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/Games/comments/1vbui6a/amd_is_reportedly_raising_graphics_card_pricesit/</t>
+          <t>https://www.gamedeveloper.com/business/how-a-surge-in-memory-prices-will-affect-the-games-industry</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update the data to the workbook of 2026-09-07
874 sources, 10 markets, 37 trends, 33 platforms, 30 genres.

Copied from public/downloads/ by scripts/build-mirror.mjs in the site
repository. Every count in the README is read from data/downloads.json rather
than typed, so it describes the files beside it.
</commit_message>
<xml_diff>
--- a/games-research-starter-pack.xlsx
+++ b/games-research-starter-pack.xlsx
@@ -474,7 +474,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Compiled from the research workbook of 2026-09-06. https://games.thisisdelightful.com</t>
+          <t>Compiled from the research workbook of 2026-09-07. https://games.thisisdelightful.com</t>
         </is>
       </c>
     </row>
@@ -55253,22 +55253,22 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Sustained mass layoffs since 2022: crowd-sourced trackers recorded ~8,500 job losses in 2022, 10,500 in 2023, and 14,600 in 2024, with ~4,000 by mid-2025 as the pace slowed. Studio closures and cancellations continued into 2026.</t>
+          <t>Sustained mass layoffs since 2022: crowd-sourced trackers recorded ~8,500 job losses in 2022, 10,500 in 2023, 14,600 in 2024 and 9,175 in 2025. The pace did not hold there. Satvat's tracker counted 10,140 confirmed losses by 11 August 2026 — past the whole of 2025 with four months left — and lifted its year-end forecast to 14,666, up about 83% from the 8,025 it projected on 6 January and just under 2024's record 15,631. Treat the forecast as one tracker's projection; the confirmed count is the firmer number. Two trackers run: Satvat's, the count quoted here, and Farhan Noor's videogamelayoffs.com, which counts differently and updates less often, so name which tracker a figure comes from.</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Nearly every business, labor, and creative-risk story of 2023 to 2026 traces back to this contraction. Indispensable for context, as it informs almost everything else.</t>
+          <t>Nearly every business, labor, and creative-risk story of 2023 to 2026 traces back to this contraction. Indispensable for context, as it informs almost everything else. Note that the 2025 dip was widely read at the time as the end of the era; 2026 says it was a trough, so date any “layoffs are slowing” claim before repeating it.</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>Game Developer's business desk, GDC State of the Game Industry (annual), Farhan Noor's videogamelayoffs.com tracker, GamesIndustry.biz</t>
+          <t>Game Developer's business desk, GDC State of the Game Industry (annual), Satvat's layoff tracker, Farhan Noor's videogamelayoffs.com tracker, GamesIndustry.biz</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>Aug 2026</t>
+          <t>Sep 2026</t>
         </is>
       </c>
     </row>
@@ -55421,7 +55421,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Game Pass is reportedly down to about 30 million paying subscribers, against an internal projection of ~77 million by 2026 revealed in FTC proceedings, after a price hike to $30/month drove churn. Sony has stopped reporting PS Plus subscriber counts.</t>
+          <t>Game Pass is reportedly down to about 30 million paying subscribers, against an internal projection of ~77 million by 2026 revealed in FTC proceedings, after a price hike to $30/month drove churn. Sony has stopped reporting PS Plus subscriber counts. From November 2026 Xbox meters cloud streaming rather than bundling it: 15 hours a month on Ultimate, 10 on Premium, 5 on Essential, with extra hours sold separately. Microsoft puts the affected share at 4% of subscribers.</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -55436,7 +55436,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>Jul 2026</t>
+          <t>Sep 2026</t>
         </is>
       </c>
     </row>
@@ -55841,7 +55841,7 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Saudi Arabia's PIF has assembled a layered gaming portfolio (Savvy, Scopely, ESL FACEIT, listed stakes) capped by taking EA private, closed August 2026. PIF holds 93.4% directly, held outside Savvy alongside Silver Lake and Affinity Partners. Roughly $20B of purchase debt now sits on EA's own books, so the debate has shifted from sportswashing and esports capture toward layoffs, cancelled projects, and quiet self-censorship.</t>
+          <t>Saudi Arabia's PIF has assembled a layered gaming portfolio (Savvy, Scopely, ESL FACEIT, listed stakes) capped by taking EA private, closed August 2026. PIF holds 93.4% directly, held outside Savvy alongside Silver Lake and Affinity Partners. Roughly $20B of purchase debt now sits on EA's own books, so the debate has shifted from sportswashing and esports capture toward layoffs, cancelled projects, and quiet self-censorship. Brian Ward, who built the portfolio from 2021, stepped down as Savvy's CEO on 1 September 2026, twelve days after the EA deal closed; PIF deputy governor Turqi Alnowaiser took over on an interim basis, moving day-to-day control closer to the fund.</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
@@ -55856,7 +55856,7 @@
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>Jul 2026</t>
+          <t>Sep 2026</t>
         </is>
       </c>
     </row>
@@ -56093,7 +56093,7 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Courts are unwinding app-store control asymmetrically. Google, having lost on all counts, must carry rival stores inside Play/ Aptoide arrived in August, and a judge ordered install friction stripped within a week. Apple, having won most counts, is re-pricing rather than losing commissions: tiered external-link fees in the US, a flat 5% replacing the EU's Core Technology Fee. Enforcement is now continuous.</t>
+          <t>Courts are unwinding app-store control asymmetrically. Google, having lost on all counts, must carry rival stores inside Play/ Aptoide arrived in August, and a judge ordered install friction stripped within a week. Apple, having won most counts, is re-pricing rather than losing commissions: tiered external-link fees in the US, a flat 5% replacing the EU's Core Technology Fee. Enforcement is now continuous. Japan moved by statute rather than by court: the Mobile Software Competition Act took full effect on 18 December 2025, and Apple's Japan changes of the day before opened iOS to rival marketplaces and outside payments, with App Store commissions cut to 10% or 21%.</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -56103,7 +56103,7 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>The Verge policy desk, MacRumors legal coverage, mobilegamer.biz, European Commission DMA enforcement updates</t>
+          <t>The Verge policy desk, MacRumors legal coverage, mobilegamer.biz, European Commission DMA enforcement updates, Japan Fair Trade Commission MSCA enforcement</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
@@ -56887,22 +56887,18 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>WTF Is Happening To The Video Game Industry?</t>
+          <t>Amir Satvat: Layoffs in the Gaming Industry in 2026</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Analysis</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr"/>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=Sx-lddna-qg</t>
+          <t>https://gamedevreports.substack.com/p/amir-satvat-layoffs-in-the-gaming</t>
         </is>
       </c>
     </row>
@@ -57167,18 +57163,18 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Game pass Subscription Coming to an End</t>
+          <t>Xbox introduces cloud streaming limits for Game Pass, purchase options for ad-hoc use</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Community</t>
+          <t>Reporting</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr"/>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/XboxGamePass/comments/1vn4rxr/game_pass_subscription_coming_to_an_end/</t>
+          <t>https://thisweekinvideogames.com/news/xbox-introduces-cloud-streaming-limits-for-game-pass-purchase-options-for-ad-hoc-use/</t>
         </is>
       </c>
     </row>
@@ -57873,18 +57869,18 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>'Hard to feel good about being bought out by a regime that's very much at odds with progressive society'</t>
+          <t>Saudi video game giant Savvy CEO Brian Ward is stepping down</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Community</t>
+          <t>Reporting</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr"/>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/gaming/comments/1vsviuy/ea_employees_brace_for_the_worst_under_saudi/</t>
+          <t>https://www.bloomberg.com/news/articles/2026-09-01/saudi-video-game-giant-savvy-ceo-brian-ward-is-stepping-down</t>
         </is>
       </c>
     </row>
@@ -58233,7 +58229,7 @@
       <c r="D61" s="3" t="inlineStr"/>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/Android/comments/1vnvxod/that_is_not_acceptable_judge_orders_google_to/</t>
+          <t>https://www.theverge.com/policy/979852/that-is-not-acceptable-judge-orders-google-to-make-rival-app-store-installs-easier</t>
         </is>
       </c>
     </row>
@@ -58245,7 +58241,7 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>Apple just rewrote its App Store fees in the EU</t>
+          <t>Apple announces changes to iOS in Japan</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
@@ -58253,14 +58249,10 @@
           <t>Community</t>
         </is>
       </c>
-      <c r="D62" s="3" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
+      <c r="D62" s="3" t="inlineStr"/>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@bigcribs/video/7675512577903938837</t>
+          <t>https://www.apple.com/newsroom/2025/12/apple-announces-changes-to-ios-in-japan/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update the data to the workbook of 2026-09-09
887 sources, 10 markets, 37 trends, 35 platforms, 30 genres.

Copied from public/downloads/ by scripts/build-mirror.mjs in the site
repository. Every count in the README is read from data/downloads.json rather
than typed, so it describes the files beside it.
</commit_message>
<xml_diff>
--- a/games-research-starter-pack.xlsx
+++ b/games-research-starter-pack.xlsx
@@ -20,7 +20,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sources'!$A$1:$R$888</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Trends'!$A$1:$H$38</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Trend reading'!$A$1:$E$110</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Trend reading'!$A$1:$E$111</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Platforms'!$A$1:$F$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Genres'!$A$1:$E$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Example games'!$A$1:$D$91</definedName>
@@ -539,7 +539,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -56157,7 +56157,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>GTA 6 launched at $80, settling speculation about $100 base games. Only Mario Kart World, GTA 6, and Elden Ring on Switch 2 have cleared $70 — Microsoft tried and retreated to $70 after backlash. Meanwhile a RAM-driven hardware crunch pushed consoles past $600 and GPUs, monitors, and memory sharply higher. Nintendo raised Switch 2 to $500 in the US, Canada and Europe from 1 September 2026 (Japan from 25 May), citing memory and component costs, and said the new price still does not cover build cost; it put the hardware-cost impact on FY2027 earnings at about ¥100bn.</t>
+          <t>GTA 6 launched at $80, settling speculation about $100 base games. Only Mario Kart World, GTA 6, and Elden Ring on Switch 2 have cleared $70 — Microsoft tried and retreated to $70 after backlash. Meanwhile a RAM-driven hardware crunch pushed consoles past $600 and GPUs, monitors, and memory sharply higher. Nintendo raised Switch 2 to $500 in the US, Canada and Europe from 1 September 2026 (Japan from 25 May), citing memory and component costs, and said the new price still does not cover build cost; it put the hardware-cost impact on FY2027 earnings at about ¥100bn. By September the crunch was moving both ways: Framework cut its LPCAMM2 memory prices retroactively while a 10 percent Intel CPU rise was reported for October and Chinese GPU prices rose again.</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -56199,7 +56199,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Live service means games built on an ongoing content and monetization cadence rather than a one-time sale. Entrants keep failing in a crowded field: Anthem went offline in January, Highguard lasted under two months. In 2026 the retreat sharpened — Guerrilla stripped live service out of Horizon Hunters Gathering mid-development, and Amazon exited MMO publishing entirely.</t>
+          <t>Live service means games built on an ongoing content and monetization cadence rather than a one-time sale. Entrants keep failing in a crowded field: Anthem went offline in January, Highguard lasted under two months. In 2026 the retreat sharpened — Guerrilla stripped live service out of Horizon Hunters Gathering mid-development, and Amazon exited MMO publishing entirely. In September 2026 Sega said it had cancelled its Super Game, a live-service project it judged too big to reach service scale, and Riot's co-founder said the free-to-play publisher is considering premium titles.</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -56214,7 +56214,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Jul 2026</t>
+          <t>Sep 2026</t>
         </is>
       </c>
     </row>
@@ -56241,7 +56241,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Game Pass is reportedly down to about 30 million paying subscribers, against an internal projection of ~77 million by 2026 revealed in FTC proceedings, after a price hike to $30/month drove churn. Sony has stopped reporting PS Plus subscriber counts. From November 2026 Xbox meters cloud streaming rather than bundling it: 15 hours a month on Ultimate, 10 on Premium, 5 on Essential, with extra hours sold separately. Microsoft puts the affected share at 4% of subscribers.</t>
+          <t>Game Pass is reportedly down to about 30 million paying subscribers, against an internal projection of ~77 million by 2026 revealed in FTC proceedings, after a price hike to $29.99 a month in October 2025 drove churn; Microsoft rolled Ultimate back to $22.99 on 26 April 2026. Sony has stopped reporting PS Plus subscriber counts. From November 2026 Xbox meters cloud streaming rather than bundling it: 15 hours a month on Ultimate, 10 on Premium, 5 on Essential, with extra hours sold separately. Microsoft puts the affected share at 4% of subscribers. Within a week of the cloud cap Microsoft began offering lapsed and some current Ultimate subscribers 12-month discounts reported at $16 to $20 a month against list, a segmented win-back test rather than a price change.</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -56325,7 +56325,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Regulators shifted from suing Roblox to compelling it: state AG suits and a 148-case federal MDL were joined in August 2026 by a Senate Judiciary probe with a records deadline, while Australia's eSafety served transparency notices on Roblox, Minecraft, Fortnite and Steam and then extracted a court-enforceable undertaking. Roblox disputes the claims and now requires facial age estimation for chat. The mechanics followed the enforcement: Microsoft makes Australians verify age by selfie, ID or credit card before buying 18+ titles on the Xbox Store, while Ofcom and the EU tighten in parallel. Elsewhere the response is blunter, with outright blocks in Turkey, Russia, Egypt and the Gulf. And it is no longer only Roblox: Brazil suspended Discord livestreaming after a teenager's death, and a Texas judge ordered Discord age checks.</t>
+          <t>Regulators shifted from suing Roblox to compelling it: state AG suits and a 148-case federal MDL were joined in August 2026 by a Senate Judiciary probe with a records deadline, while Australia's eSafety served transparency notices on Roblox, Minecraft, Fortnite and Steam and then extracted a court-enforceable undertaking. Roblox disputes the claims and now requires facial age estimation for chat. The mechanics followed the enforcement: Microsoft makes Australians verify age by selfie, ID or credit card before buying 18+ titles on the Xbox Store; in September 2026 Steam began requiring a credit card for R18+ purchases in Australia and the Epic Games Store announced age checks for R18+ titles, while Ofcom and the EU tighten in parallel. Elsewhere the response is blunter, with outright blocks in Turkey, Russia, Egypt and the Gulf. And it is no longer only Roblox: Brazil suspended Discord livestreaming after a teenager's death, and a Texas judge ordered Discord age checks.</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -56340,7 +56340,7 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>Aug 2026</t>
+          <t>Sep 2026</t>
         </is>
       </c>
     </row>
@@ -56703,7 +56703,7 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Matthew Ball's analysis of where 2025's growth actually went: of the ~$10 billion industry increase versus 2021, about $4 billion was in China and another $1.5 billion went to China-made games in global markets, with 84% of Chinese game revenue going to domestically made games. This means that growth is concentrated in places and platforms many Western publishers can't reach.</t>
+          <t>Matthew Ball's analysis of where 2025's growth actually went: of the ~$10 billion industry increase versus 2021, about $4 billion was in China and another $1.5 billion went to China-made games in global markets, with 84% of Chinese game revenue going to domestically made games. This means that growth is concentrated in places and platforms many Western publishers can't reach. Niko Partners puts China's 2025 games revenue at $51.8 billion, up 5.4 percent and above $50 billion for the first time, with annual ARPU past $70 and mini games near a fifth of mobile spend; it forecasts $53.9 billion for 2026 and $59.8 billion by 2030.</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -56718,7 +56718,7 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>Jul 2026</t>
+          <t>Sep 2026</t>
         </is>
       </c>
     </row>
@@ -56787,7 +56787,7 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Adoption keeps rising while sentiment collapses: 52% of surveyed game professionals now say generative AI is harming the industry, up from 30% the year before and 18% the year prior, with art and narrative roles most negative. Company-level use (52%) has decoupled from individual use (36%), and the argument has moved from opinion to enforcement.</t>
+          <t>Adoption keeps rising while sentiment collapses: 52% of surveyed game professionals now say generative AI is harming the industry, up from 30% the year before and 18% the year prior, with art and narrative roles most negative. Company-level use (52%) has decoupled from individual use (36%), and the argument has moved from opinion to enforcement. A European survey by Values Value and InGame Job, reported in September 2026, found the fear is pace before replacement: 61 percent expect generative AI to push them to work faster against 35 percent who fear for their role, and 35 percent of founders say they have already declined a hire because AI could do the work.</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -56802,7 +56802,7 @@
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>Jul 2026</t>
+          <t>Sep 2026</t>
         </is>
       </c>
     </row>
@@ -56913,7 +56913,7 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Courts are unwinding app-store control asymmetrically. Google, having lost on all counts, must carry rival stores inside Play/ Aptoide arrived in August, and a judge ordered install friction stripped within a week. Apple, having won most counts, is re-pricing rather than losing commissions: tiered external-link fees in the US, a flat 5% replacing the EU's Core Technology Fee. Enforcement is now continuous. Japan moved by statute rather than by court: the Mobile Software Competition Act took full effect on 18 December 2025, and Apple's Japan changes of the day before opened iOS to rival marketplaces and outside payments, with App Store commissions cut to 10% or 21%.</t>
+          <t>Courts are unwinding app-store control asymmetrically. Google, having lost on all counts, must carry rival stores inside Play/ Aptoide arrived in August, and a judge ordered install friction stripped within a week. Apple, having won most counts, is re-pricing rather than losing commissions: tiered external-link fees in the US, a flat 5% Core Technology Commission and a 15% steering fee replacing the EU's Core Technology Fee from 18 August 2026, terms eighteen developer groups including the EGDF rejected in September as a breach of the DMA's free-steering article. Enforcement is now continuous. Japan moved by statute rather than by court: the Mobile Software Competition Act took full effect on 18 December 2025, and Apple's Japan changes of the day before opened iOS to rival marketplaces and outside payments, with App Store commissions cut to 10% or 21%.</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -56928,7 +56928,7 @@
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>Jul 2026</t>
+          <t>Sep 2026</t>
         </is>
       </c>
     </row>
@@ -57039,7 +57039,7 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>The 2021 to 2022 wave of metaverse platforms and NFT/play-to-earn games has largely collapsed or rebranded. Matthew Ball's retrospective analysis groups web3 among growth engines that failed to deliver on their hype, leaving the industry stalled. Persistent worlds and UGC ideas have survived inside Roblox/Fortnite, but the token economics mostly did not.</t>
+          <t>The 2021 to 2022 wave of metaverse platforms and NFT/play-to-earn games has largely collapsed or rebranded. Matthew Ball's retrospective analysis groups web3 among growth engines that failed to deliver on their hype, leaving the industry stalled. Persistent worlds and UGC ideas have survived inside Roblox/Fortnite, but the token economics mostly did not. The exceptions are publisher-backed: Nexon's NEXPACE reported 30.98 million NXPC of first-half 2026 protocol revenue from MapleStory Universe, a running token economy inside a live IP.</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
@@ -57054,7 +57054,7 @@
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>Jul 2026</t>
+          <t>Sep 2026</t>
         </is>
       </c>
     </row>
@@ -57123,7 +57123,7 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>A long-running argument about whether buying a game confers ownership, reignited each time a publisher shuts down servers and renders a purchased title unplayable. Its most visible chapter, Stop Killing Games, gathered 1,294,188 verified signatures across 24 EU member states. On 16 June 2026 the Commission declined to propose a legal obligation, citing intellectual property constraints, offering a voluntary industry code of conduct instead; the campaign has pivoted to amending the Digital Fairness Act, due Q4 2026. The fight has since globalised into three tracks. Legislation: Brazil's PL 3612/2026 would mandate point-of-sale disclosure of server dependence, a two-year minimum support window, and a state preservation fund framed as digital cultural heritage. Litigation: UFC-Que Choisir is suing Ubisoft over The Crew, and a Dutch class action targets the PlayStation Store. Archives: Japan mandates legal deposit yet bars access without rightsholder consent, pushing its Game Preservation Society to open a US office. Sony's 2028 disc cutoff has pulled the question mainstream.</t>
+          <t>A long-running argument about whether buying a game confers ownership, reignited each time a publisher shuts down servers and renders a purchased title unplayable. Its most visible chapter, Stop Killing Games, gathered 1,294,188 verified signatures across 24 EU member states. On 16 June 2026 the Commission declined to propose a legal obligation, citing intellectual property constraints, offering a voluntary industry code of conduct instead; the campaign has pivoted to amending the Digital Fairness Act, due Q4 2026. The fight has since globalised into three tracks. Legislation: Brazil's PL 3612/2026 would mandate point-of-sale disclosure of server dependence, a two-year minimum support window, and a state preservation fund framed as digital cultural heritage. Litigation: UFC-Que Choisir is suing Ubisoft over The Crew, and a Dutch class action targets the PlayStation Store. Archives: Japan mandates legal deposit yet bars access without rightsholder consent, pushing its Game Preservation Society to open a US office. Sony's 2028 disc cutoff has pulled the question mainstream. In September 2026 the argument reached the console itself: Xbox's Disc-to-Digital, which converts a disc into a digital licence, launched to Insiders with Sega, Square Enix, Ubisoft and Bandai Namco discs returning "not participating", while GOG began printing big-box artwork under its preservation programme.</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
@@ -57138,7 +57138,7 @@
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>Jul 2026</t>
+          <t>Sep 2026</t>
         </is>
       </c>
     </row>
@@ -57165,7 +57165,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Union drives hardened into institutions during the layoff era: 82% of US-based respondents to GDC's 2026 survey support unionisation, and one in four were laid off in the last two years. Microsoft's studios host the largest US unions and CWA's direct-join model now recruits across employers. Six European unions signed a cross-border action plan; France struck nationally. Nordic sectoral agreements remain the mature template.</t>
+          <t>Union drives hardened into institutions during the layoff era: 82% of US-based respondents to GDC's 2026 survey support unionisation, and one in four were laid off in the last two years. Microsoft's studios host the largest US unions and CWA's direct-join model now recruits across employers. Six European unions signed a cross-border action plan; France struck nationally. Nordic sectoral agreements remain the mature template. In September 2026 about 1,900 Blizzard workers ratified a CWA master contract with layoff recall rights, four extra weeks of severance and a duty on Microsoft to bargain over AI use, while the final tribunal hearing over Rockstar North's dismissal of union members opened in the UK.</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -57180,7 +57180,7 @@
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>Jul 2026</t>
+          <t>Sep 2026</t>
         </is>
       </c>
     </row>
@@ -57249,7 +57249,7 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>The VC money is gone and the correction is over — this is the aftermath. What's left is a two-pillar economy: publisher-run circuits and Saudi-funded events (Esports World Cup, $75m prize pool, ~$20m distributed to 40 partner clubs). Global revenue is ~$5.34b and growing, but teams are the weakest link. Break-even is now a headline achievement, not a baseline: DRX is filing for a Singapore listing on the strength of $8.6m revenue and two consecutive break-even years. Franchising starts unwinding into open qualifiers in 2027.</t>
+          <t>The VC money is gone and the correction is over — this is the aftermath. What's left is a two-pillar economy: publisher-run circuits and Saudi-funded events (Esports World Cup, $75m prize pool, ~$20m distributed to 40 partner clubs). Global revenue is ~$5.34b and growing, but teams are the weakest link. Break-even is now a headline achievement, not a baseline: DRX is filing for a Singapore listing on the strength of $8.6m revenue and two consecutive break-even years. Franchising starts unwinding into open qualifiers in 2027. Streams Charts' read of EWC 2026's co-streams put India first by hours watched at 12.2 percent, the top three countries only 32 percent combined and English 30 percent of the language mix, before an audience 89 percent male and a third aged 20 to 24.</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
@@ -57264,7 +57264,7 @@
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>Jul 2026</t>
+          <t>Sep 2026</t>
         </is>
       </c>
     </row>
@@ -57501,7 +57501,7 @@
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>New releases take 12 to 13% of total player time across PC and console and have for three years, with Xbox highest at 18% on Game Pass availability. Playtime is concentrated, 80% of it in 79 games on PC, 74 on PlayStation and 91 on Xbox, but that concentration loosened in 2025 and PC playtime growth since 2022 has come entirely from titles outside the top 20. Price architecture differs sharply: 76 to 79% of console revenue comes from games above $50, while PC splits near-evenly across sub-$30, $30 to $50 and above.</t>
+          <t>New releases take 12 to 13% of total player time across PC and console and have for three years, with Xbox highest at 18% on Game Pass availability. Playtime is concentrated, 80% of it in 79 games on PC, 74 on PlayStation and 91 on Xbox, but that concentration loosened in 2025 and PC playtime growth since 2022 has come entirely from titles outside the top 20. Price architecture differs sharply: 76 to 79% of console revenue comes from games above $50, while PC splits near-evenly across sub-$30, $30 to $50 and above. On the money side, Alinea Analytics estimates Steam took more than $15 billion gross in the first eight months of 2026 with the top 100 new 2026 releases about 16 percent of it, Forza Horizon 6 the largest at roughly $210 million.</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
@@ -57516,7 +57516,7 @@
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>Aug 2026</t>
+          <t>Sep 2026</t>
         </is>
       </c>
     </row>
@@ -57616,7 +57616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E110"/>
+  <dimension ref="A1:E111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="54" customWidth="1" min="1" max="1"/>
@@ -57914,18 +57914,18 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Market saturation is an excuse when level design sucks</t>
+          <t>Sega cancelled its "risky" Super Game project</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Community</t>
+          <t>Reporting</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr"/>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/gamedev/comments/1vgg93n/stop_using_market_saturation_as_an_excuse_for/</t>
+          <t>https://www.gamesindustry.biz/sega-cancelled-its-risky-super-game-project-as-it-would-have-to-grow-enormously-to-match-the-scale-of-the-service</t>
         </is>
       </c>
     </row>
@@ -58121,18 +58121,18 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Xbox lets 'longstanding' accounts bypass age verification checks</t>
+          <t>Steam implements age verification for R18+ games in Australia, credit card required</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Community</t>
+          <t>Reporting</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr"/>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/pcgaming/comments/1vlorr7/xbox_lets_longstanding_accounts_bypass_age/</t>
+          <t>https://thisweekinvideogames.com/news/steam-implements-age-verification-for-r18-games-in-australia-credit-card-required/</t>
         </is>
       </c>
     </row>
@@ -58730,23 +58730,23 @@
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>China's banhao throttles games</t>
+          <t>Western publishers can't access Chinese growth</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>Niko Partners, analyst research note, Jan 2026</t>
+          <t>Chinese gaming market surpasses $50 billion</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Analysis</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr"/>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>https://substack.nikopartners.com/p/chinas-nppa-approved-1771-video-games</t>
+          <t>https://nikopartners.com/chinese-gaming-market-surpasses-50-billion-as-ai-premium-gaming-and-new-monetization-models-reshape-growth/</t>
         </is>
       </c>
     </row>
@@ -58758,18 +58758,18 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>Chinese gacha games recorded an 8.97% decline, despite growth in the gaming industry as a whole</t>
+          <t>Niko Partners, analyst research note, Jan 2026</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Community</t>
+          <t>Analysis</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr"/>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/gachagaming/comments/1vauysu/china_game_industry_report_for_januaryjune_2026/</t>
+          <t>https://substack.nikopartners.com/p/chinas-nppa-approved-1771-video-games</t>
         </is>
       </c>
     </row>
@@ -58781,30 +58781,30 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>China Game Approval (Banhao) requirements for apps in CN, 2026</t>
+          <t>Chinese gacha games recorded an 8.97% decline, despite growth in the gaming industry as a whole</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>Primary</t>
+          <t>Community</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr"/>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>https://clearlaunch.dev/regulations/china-game-approval</t>
+          <t>https://www.reddit.com/r/gachagaming/comments/1vauysu/china_game_industry_report_for_januaryjune_2026/</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>Generative AI in development: the enforcement turn</t>
+          <t>China's banhao throttles games</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>GDC 2026 State of the Game Industry Reveals Impact of Layoffs, Generative AI, and More</t>
+          <t>China Game Approval (Banhao) requirements for apps in CN, 2026</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
@@ -58815,7 +58815,7 @@
       <c r="D51" s="3" t="inlineStr"/>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>https://gdconf.com/article/gdc-2026-state-of-the-game-industry-reveals-impact-of-layoffs-generative-ai-and-more/</t>
+          <t>https://clearlaunch.dev/regulations/china-game-approval</t>
         </is>
       </c>
     </row>
@@ -58827,18 +58827,18 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>AI is a copyright landmine: "I think we're going to see lawsuits"</t>
+          <t>GDC 2026 State of the Game Industry Reveals Impact of Layoffs, Generative AI, and More</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Analysis</t>
+          <t>Primary</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr"/>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>https://www.gamesradar.com/games/echoing-palworld-dev-video-game-lawyer-says-all-her-clients-have-anti-ai-contracts-because-gamers-hate-it-and-its-a-copyright-landmine-i-think-were-going-to-see-lawsuits/</t>
+          <t>https://gdconf.com/article/gdc-2026-state-of-the-game-industry-reveals-impact-of-layoffs-generative-ai-and-more/</t>
         </is>
       </c>
     </row>
@@ -58850,41 +58850,41 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>r/gamedev Policy on AI Use</t>
+          <t>AI is a copyright landmine: "I think we're going to see lawsuits"</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Community</t>
+          <t>Analysis</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr"/>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/gamedev/comments/1vrnqyt/rgamedev_policy_on_ai_use/</t>
+          <t>https://www.gamesradar.com/games/echoing-palworld-dev-video-game-lawyer-says-all-her-clients-have-anti-ai-contracts-because-gamers-hate-it-and-its-a-copyright-landmine-i-think-were-going-to-see-lawsuits/</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>The rise of AI companions &amp; co-playable NPCs</t>
+          <t>Generative AI in development: the enforcement turn</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>How KRAFTON Built PUBG Ally, a Co-Playable Character Powered by NVIDIA ACE</t>
+          <t>European game developers are more concerned that AI will pressure them to work faster rather than take their job</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>Analysis</t>
+          <t>Reporting</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr"/>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>https://developer.nvidia.com/blog/how-krafton-built-pubg-ally-a-co-playable-character-powered-by-nvidia-ace/</t>
+          <t>https://www.gamesindustry.biz/european-game-developers-are-more-concerned-that-ai-will-pressure-them-to-work-faster-rather-than-take-their-job</t>
         </is>
       </c>
     </row>
@@ -58896,18 +58896,18 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>r/gamedev Policy on AI Use</t>
+          <t>How KRAFTON Built PUBG Ally, a Co-Playable Character Powered by NVIDIA ACE</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>Community</t>
+          <t>Analysis</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr"/>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/gamedev/comments/1vrnqyt/rgamedev_policy_on_ai_use/</t>
+          <t>https://developer.nvidia.com/blog/how-krafton-built-pubg-ally-a-co-playable-character-powered-by-nvidia-ace/</t>
         </is>
       </c>
     </row>
@@ -58919,7 +58919,7 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>dev stress-tests their game's voice recognition after a player calls it bad</t>
+          <t>r/gamedev Policy on AI Use</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
@@ -58927,37 +58927,37 @@
           <t>Community</t>
         </is>
       </c>
-      <c r="D56" s="3" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
+      <c r="D56" s="3" t="inlineStr"/>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@monchiistudio/video/7676265366301019393</t>
+          <t>https://www.reddit.com/r/gamedev/comments/1vrnqyt/rgamedev_policy_on_ai_use/</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>Who the AI agreement left out</t>
+          <t>The rise of AI companions &amp; co-playable NPCs</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>SAG-AFTRA Overwhelmingly Approves Video Game Agreement, Marking Official End To Nearly Yearlong Strike</t>
+          <t>dev stress-tests their game's voice recognition after a player calls it bad</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>Reporting</t>
-        </is>
-      </c>
-      <c r="D57" s="3" t="inlineStr"/>
+          <t>Community</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>https://deadline.com/2025/07/sag-aftra-video-game-agreement-approved-strike-1236453741/</t>
+          <t>https://www.tiktok.com/@monchiistudio/video/7676265366301019393</t>
         </is>
       </c>
     </row>
@@ -58969,7 +58969,7 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>Saber's AI Rideshare Stimulator controversy almost closes on high note</t>
+          <t>SAG-AFTRA Overwhelmingly Approves Video Game Agreement, Marking Official End To Nearly Yearlong Strike</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
@@ -58980,7 +58980,7 @@
       <c r="D58" s="3" t="inlineStr"/>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>https://www.pcgamer.com/gaming-industry/sabers-ai-rideshare-stimulator-controversy-almost-closes-on-high-note-with-ceo-apology-then-he-calls-portal-scribe-who-mocked-him-an-unsuccessful-writer/</t>
+          <t>https://deadline.com/2025/07/sag-aftra-video-game-agreement-approved-strike-1236453741/</t>
         </is>
       </c>
     </row>
@@ -58992,7 +58992,7 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>Video game lawyer says all her clients have anti-AI contracts because gamers hate it</t>
+          <t>Saber's AI Rideshare Stimulator controversy almost closes on high note</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
@@ -59003,19 +59003,19 @@
       <c r="D59" s="3" t="inlineStr"/>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>https://www.gamesradar.com/games/echoing-palworld-dev-video-game-lawyer-says-all-her-clients-have-anti-ai-contracts-because-gamers-hate-it-and-its-a-copyright-landmine-i-think-were-going-to-see-lawsuits/</t>
+          <t>https://www.pcgamer.com/gaming-industry/sabers-ai-rideshare-stimulator-controversy-almost-closes-on-high-note-with-ceo-apology-then-he-calls-portal-scribe-who-mocked-him-an-unsuccessful-writer/</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>App stores are unbundling under court supervision</t>
+          <t>Who the AI agreement left out</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>Following Epic loss, Google has started hosting rival app stores in Play Store</t>
+          <t>Video game lawyer says all her clients have anti-AI contracts because gamers hate it</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
@@ -59026,7 +59026,7 @@
       <c r="D60" s="3" t="inlineStr"/>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>https://arstechnica.com/gadgets/2026/08/third-party-app-stores-are-rolling-out-in-google-play-but-theres-only-one-right-now/</t>
+          <t>https://www.gamesradar.com/games/echoing-palworld-dev-video-game-lawyer-says-all-her-clients-have-anti-ai-contracts-because-gamers-hate-it-and-its-a-copyright-landmine-i-think-were-going-to-see-lawsuits/</t>
         </is>
       </c>
     </row>
@@ -59038,18 +59038,18 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>'That is not acceptable': Judge orders Google to make rival app store installs easier</t>
+          <t>Following Epic loss, Google has started hosting rival app stores in Play Store</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>Community</t>
+          <t>Reporting</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr"/>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>https://www.theverge.com/policy/979852/that-is-not-acceptable-judge-orders-google-to-make-rival-app-store-installs-easier</t>
+          <t>https://arstechnica.com/gadgets/2026/08/third-party-app-stores-are-rolling-out-in-google-play-but-theres-only-one-right-now/</t>
         </is>
       </c>
     </row>
@@ -59061,7 +59061,7 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>Apple announces changes to iOS in Japan</t>
+          <t>'That is not acceptable': Judge orders Google to make rival app store installs easier</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
@@ -59072,30 +59072,30 @@
       <c r="D62" s="3" t="inlineStr"/>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>https://www.apple.com/newsroom/2025/12/apple-announces-changes-to-ios-in-japan/</t>
+          <t>https://www.theverge.com/policy/979852/that-is-not-acceptable-judge-orders-google-to-make-rival-app-store-installs-easier</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>Streamers fragment across platforms</t>
+          <t>App stores are unbundling under court supervision</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>Multistreaming Audience Split: Twitch, YouTube &amp; Kick in H1 2026</t>
+          <t>Apple announces changes to iOS in Japan</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Community</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr"/>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>https://streamscharts.com/news/multistreaming-audience-split-twitch-youtube-kick-h1-2026</t>
+          <t>https://www.apple.com/newsroom/2025/12/apple-announces-changes-to-ios-in-japan/</t>
         </is>
       </c>
     </row>
@@ -59107,7 +59107,7 @@
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>SOOP Korea and Chzzk: One Year After Twitch's Shutdown</t>
+          <t>Multistreaming Audience Split: Twitch, YouTube &amp; Kick in H1 2026</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
@@ -59118,7 +59118,7 @@
       <c r="D64" s="3" t="inlineStr"/>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>https://streamhatchet.com/blog/the-state-of-korean-live-streaming/</t>
+          <t>https://streamscharts.com/news/multistreaming-audience-split-twitch-youtube-kick-h1-2026</t>
         </is>
       </c>
     </row>
@@ -59130,41 +59130,41 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>Twitch now uses channel VODs, clips and chat messages to train generative AI by default</t>
+          <t>SOOP Korea and Chzzk: One Year After Twitch's Shutdown</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>Community</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr"/>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/LivestreamFail/comments/1vmnkfz/twitch_now_uses_channel_vods_clips_and_chat/</t>
+          <t>https://streamhatchet.com/blog/the-state-of-korean-live-streaming/</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>Handheld PC resurgence</t>
+          <t>Streamers fragment across platforms</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>Asus ROG Xbox Ally sales stall with Steam Deck still the preferred handheld gaming PC</t>
+          <t>Twitch now uses channel VODs, clips and chat messages to train generative AI by default</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>Reporting</t>
+          <t>Community</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr"/>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>https://www.notebookcheck.net/Asus-ROG-Xbox-Ally-sales-stall-with-Steam-Deck-still-the-preferred-handheld-gaming-PC.1230155.0.html</t>
+          <t>https://www.reddit.com/r/LivestreamFail/comments/1vmnkfz/twitch_now_uses_channel_vods_clips_and_chat/</t>
         </is>
       </c>
     </row>
@@ -59176,18 +59176,18 @@
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>SteamOS expands beyond Steam Deck</t>
+          <t>Asus ROG Xbox Ally sales stall with Steam Deck still the preferred handheld gaming PC</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>Primary</t>
+          <t>Reporting</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr"/>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>https://store.steampowered.com/news/app/593110/view/529834914570306831</t>
+          <t>https://www.notebookcheck.net/Asus-ROG-Xbox-Ally-sales-stall-with-Steam-Deck-still-the-preferred-handheld-gaming-PC.1230155.0.html</t>
         </is>
       </c>
     </row>
@@ -59199,45 +59199,45 @@
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>PC Gaming Handhelds just keep getting better</t>
+          <t>SteamOS expands beyond Steam Deck</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>Community</t>
-        </is>
-      </c>
-      <c r="D68" s="3" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
+          <t>Primary</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr"/>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@gg.sheed/video/7675986246526700814</t>
+          <t>https://store.steampowered.com/news/app/593110/view/529834914570306831</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>Metaverse &amp; blockchain gaming hype</t>
+          <t>Handheld PC resurgence</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>Matthew Ball / Epyllion, industry report, May 2026</t>
+          <t>PC Gaming Handhelds just keep getting better</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>Analysis</t>
-        </is>
-      </c>
-      <c r="D69" s="3" t="inlineStr"/>
+          <t>Community</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>https://www.matthewball.co/all/presentation-the-state-of-video-gaming-in-2026</t>
+          <t>https://www.tiktok.com/@gg.sheed/video/7675986246526700814</t>
         </is>
       </c>
     </row>
@@ -59249,7 +59249,7 @@
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>More than 90% of Web3 games failed after $15 billion boom</t>
+          <t>Matthew Ball / Epyllion, industry report, May 2026</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
@@ -59260,7 +59260,7 @@
       <c r="D70" s="3" t="inlineStr"/>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>https://www.coindesk.com/markets/2026/04/23/more-than-90-of-web3-games-failed-after-usd15-billion-boom-as-gamers-never-showed-up-caladan</t>
+          <t>https://www.matthewball.co/all/presentation-the-state-of-video-gaming-in-2026</t>
         </is>
       </c>
     </row>
@@ -59272,41 +59272,41 @@
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>Stablecoins Gain Ground in Blockchain Gaming as Studios Tighten Spending, Study Finds</t>
+          <t>More than 90% of Web3 games failed after $15 billion boom</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>Reporting</t>
+          <t>Analysis</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr"/>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>https://finance.yahoo.com/news/stablecoins-gain-ground-blockchain-gaming-023901223.html</t>
+          <t>https://www.coindesk.com/markets/2026/04/23/more-than-90-of-web3-games-failed-after-usd15-billion-boom-as-gamers-never-showed-up-caladan</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>Gaming is now cross-generational</t>
+          <t>Metaverse &amp; blockchain gaming hype</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>2026 Essential Facts About the U.S. Video Game Industry</t>
+          <t>NEXPACE posts 30.98 million NXPC in first-half protocol revenue</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Reporting</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr"/>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>https://www.theesa.com/resources/essential-facts-about-the-us-video-game-industry/2026-data/</t>
+          <t>https://www.invenglobal.com/articles/25725/nexpace-posts-3098-million-nxpc-in-first-half-protocol-revenue</t>
         </is>
       </c>
     </row>
@@ -59318,22 +59318,18 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>The Myth of the Aging Playerbase</t>
+          <t>2026 Essential Facts About the U.S. Video Game Industry</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>Analysis</t>
-        </is>
-      </c>
-      <c r="D73" s="3" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr"/>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=N8tdqi-x9OI</t>
+          <t>https://www.theesa.com/resources/essential-facts-about-the-us-video-game-industry/2026-data/</t>
         </is>
       </c>
     </row>
@@ -59345,7 +59341,7 @@
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>Why older gamers could be the key to saving the games industry</t>
+          <t>The Myth of the Aging Playerbase</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
@@ -59353,33 +59349,37 @@
           <t>Analysis</t>
         </is>
       </c>
-      <c r="D74" s="3" t="inlineStr"/>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
       <c r="E74" s="3" t="inlineStr">
         <is>
-          <t>https://news.northeastern.edu/2026/06/02/old-gamers-video-game-industry/</t>
+          <t>https://www.youtube.com/watch?v=N8tdqi-x9OI</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>Players fight for digital preservation</t>
+          <t>Gaming is now cross-generational</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>Stop Destroying Videogames - Commission's reply to the European citizens' initiative</t>
+          <t>Why older gamers could be the key to saving the games industry</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>Primary</t>
+          <t>Analysis</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr"/>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>https://citizens-initiative.europa.eu/stop-destroying-videogames-commissions-reply-european-citizens-initiative_en</t>
+          <t>https://news.northeastern.edu/2026/06/02/old-gamers-video-game-industry/</t>
         </is>
       </c>
     </row>
@@ -59391,18 +59391,18 @@
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>When did StopKillingGames turn into WeWantPhysical</t>
+          <t>Stop Destroying Videogames - Commission's reply to the European citizens' initiative</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>Community</t>
+          <t>Primary</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr"/>
       <c r="E76" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/StopKillingGames/comments/1vri0w0/when_did_stopkillinggames_turn_into_wewantphysical/</t>
+          <t>https://citizens-initiative.europa.eu/stop-destroying-videogames-commissions-reply-european-citizens-initiative_en</t>
         </is>
       </c>
     </row>
@@ -59414,7 +59414,7 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>Projeto de lei inspirado no Stop Killing Games é apresentado no Brasil para evitar que jogos morram</t>
+          <t>GOG brings back "big box" PC games, one printable template at a time</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
@@ -59425,30 +59425,30 @@
       <c r="D77" s="3" t="inlineStr"/>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>https://www.tecmundo.com.br/voxel/504819-projeto-de-lei-inspirado-no-stop-killing-games-e-apresentado-no-brasil-para-evitar-que-jogos-morram.htm</t>
+          <t>https://arstechnica.com/gaming/2026/09/gog-brings-back-big-box-pc-games-one-printable-template-at-a-time/</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>Game labor is organizing</t>
+          <t>Players fight for digital preservation</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>Game Worker Solidarity: Mapping and documenting collective movements by game workers</t>
+          <t>Projeto de lei inspirado no Stop Killing Games é apresentado no Brasil para evitar que jogos morram</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>Primary</t>
+          <t>Reporting</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr"/>
       <c r="E78" s="3" t="inlineStr">
         <is>
-          <t>https://gameworkersolidarity.com/</t>
+          <t>https://www.tecmundo.com.br/voxel/504819-projeto-de-lei-inspirado-no-stop-killing-games-e-apresentado-no-brasil-para-evitar-que-jogos-morram.htm</t>
         </is>
       </c>
     </row>
@@ -59460,7 +59460,7 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>One industry, one fight – Video Game Unions Present a United Front Across Western Europe</t>
+          <t>Game Worker Solidarity: Mapping and documenting collective movements by game workers</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
@@ -59471,7 +59471,7 @@
       <c r="D79" s="3" t="inlineStr"/>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t>https://www.stjv.fr/en/2025/12/one-industry-one-fight-video-game-unions-present-a-united-front-across-western-europe/</t>
+          <t>https://gameworkersolidarity.com/</t>
         </is>
       </c>
     </row>
@@ -59483,41 +59483,41 @@
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>Rockstar faces union busting allegations</t>
+          <t>One industry, one fight – Video Game Unions Present a United Front Across Western Europe</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>Reporting</t>
+          <t>Primary</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr"/>
       <c r="E80" s="3" t="inlineStr">
         <is>
-          <t>https://www.pcgamer.com/gaming-industry/rockstar-faces-legal-setback-as-uk-tribunal-allows-its-fired-workers-to-bring-every-one-of-their-union-busting-allegations-to-trial/</t>
+          <t>https://www.stjv.fr/en/2025/12/one-industry-one-fight-video-game-unions-present-a-united-front-across-western-europe/</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>The gaming culture war continues</t>
+          <t>Game labor is organizing</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>Forced: Perceptions of “Woke” Politics in Video Games</t>
+          <t>Blizzard union workers ratify historic contract covering 1,900 employees</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Reporting</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr"/>
       <c r="E81" s="3" t="inlineStr">
         <is>
-          <t>https://ijoc.org/index.php/ijoc/article/view/23165</t>
+          <t>https://www.gamedeveloper.com/production/blizzard-union-workers-ratify-historic-contract-covering-1-900-employees</t>
         </is>
       </c>
     </row>
@@ -59529,18 +59529,18 @@
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>Steam review bombing is gaming's most powerful method of protest</t>
+          <t>Forced: Perceptions of “Woke” Politics in Video Games</t>
         </is>
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>Reporting</t>
+          <t>Research</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr"/>
       <c r="E82" s="3" t="inlineStr">
         <is>
-          <t>https://www.pcgamer.com/games/third-person-shooter/steam-review-bombing-is-gamings-most-powerful-method-of-protest-3-takeaways-from-helldivers-2s-weekend-meltdown/</t>
+          <t>https://ijoc.org/index.php/ijoc/article/view/23165</t>
         </is>
       </c>
     </row>
@@ -59552,41 +59552,41 @@
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>I hate what the culture wars have done to the discourse surrounding this game</t>
+          <t>Steam review bombing is gaming's most powerful method of protest</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>Community</t>
+          <t>Reporting</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr"/>
       <c r="E83" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/ShitHaloSays/comments/1vaslzl/i_hate_what_the_culture_wars_have_done_to_the/</t>
+          <t>https://www.pcgamer.com/games/third-person-shooter/steam-review-bombing-is-gamings-most-powerful-method-of-protest-3-takeaways-from-helldivers-2s-weekend-meltdown/</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>Esports after the reckoning</t>
+          <t>The gaming culture war continues</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>Esports Business H1 2026: 4 Shifts Reshaping the Industry</t>
+          <t>I hate what the culture wars have done to the discourse surrounding this game</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>Analysis</t>
+          <t>Community</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr"/>
       <c r="E84" s="3" t="inlineStr">
         <is>
-          <t>https://escharts.com/news/esports-business-h1-2026</t>
+          <t>https://www.reddit.com/r/ShitHaloSays/comments/1vaslzl/i_hate_what_the_culture_wars_have_done_to_the/</t>
         </is>
       </c>
     </row>
@@ -59598,18 +59598,18 @@
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>Kiwoom aims to become the first publicly listed Korean eSports team</t>
+          <t>Esports Business H1 2026: 4 Shifts Reshaping the Industry</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>Community</t>
+          <t>Analysis</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr"/>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/leagueoflegends/comments/1v46rdr/investchosun_kiwoom_drx_krx_files_for_ipo_on_the/</t>
+          <t>https://escharts.com/news/esports-business-h1-2026</t>
         </is>
       </c>
     </row>
@@ -59621,7 +59621,7 @@
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>First Esports Nations Cup delayed until 2027</t>
+          <t>Kiwoom aims to become the first publicly listed Korean eSports team</t>
         </is>
       </c>
       <c r="C86" s="3" t="inlineStr">
@@ -59629,37 +59629,33 @@
           <t>Community</t>
         </is>
       </c>
-      <c r="D86" s="3" t="inlineStr">
-        <is>
-          <t>video</t>
-        </is>
-      </c>
+      <c r="D86" s="3" t="inlineStr"/>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@bbcnews/video/7675483418607619330</t>
+          <t>https://www.reddit.com/r/leagueoflegends/comments/1v46rdr/investchosun_kiwoom_drx_krx_files_for_ipo_on_the/</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>Games media captured by large corps</t>
+          <t>Esports after the reckoning</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>Aftermath (Jackson Ryan), eight-month investigation, Mar 2026</t>
+          <t>Who watched EWC 2026 co-streams? Audience demographics and key markets</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>Analysis</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr"/>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>https://aftermath.site/gameshub-clickout-media-seo-gambling-ai/</t>
+          <t>https://streamscharts.com/news/who-watched-ewc-2026-co-streams</t>
         </is>
       </c>
     </row>
@@ -59671,7 +59667,7 @@
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>our Companies Control Your Favorite Gaming Media</t>
+          <t>Aftermath (Jackson Ryan), eight-month investigation, Mar 2026</t>
         </is>
       </c>
       <c r="C88" s="3" t="inlineStr">
@@ -59682,7 +59678,7 @@
       <c r="D88" s="3" t="inlineStr"/>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>https://spilled.gg/companies-gaming-media/</t>
+          <t>https://aftermath.site/gameshub-clickout-media-seo-gambling-ai/</t>
         </is>
       </c>
     </row>
@@ -59694,7 +59690,7 @@
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>Future, Ziff Davis to Struggle Most From Traffic Drops</t>
+          <t>our Companies Control Your Favorite Gaming Media</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
@@ -59705,30 +59701,30 @@
       <c r="D89" s="3" t="inlineStr"/>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>https://www.amediaoperator.com/analysis/future-ziff-davis-to-struggle-most-from-traffic-drops/</t>
+          <t>https://spilled.gg/companies-gaming-media/</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="3" t="inlineStr">
         <is>
-          <t>Studio investment in games plummets</t>
+          <t>Games media captured by large corps</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>The State of Video Gaming in 2026 (Matthew Ball / Epyllion)</t>
+          <t>Future, Ziff Davis to Struggle Most From Traffic Drops</t>
         </is>
       </c>
       <c r="C90" s="3" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Analysis</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr"/>
       <c r="E90" s="3" t="inlineStr">
         <is>
-          <t>https://www.matthewball.co/all/presentation-the-state-of-video-gaming-in-2026</t>
+          <t>https://www.amediaoperator.com/analysis/future-ziff-davis-to-struggle-most-from-traffic-drops/</t>
         </is>
       </c>
     </row>
@@ -59740,18 +59736,18 @@
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>The state of video games with Matthew Ball – Part One</t>
+          <t>The State of Video Gaming in 2026 (Matthew Ball / Epyllion)</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>Analysis</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr"/>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>https://www.thegamebusiness.com/p/the-state-of-video-games-with-matthew</t>
+          <t>https://www.matthewball.co/all/presentation-the-state-of-video-gaming-in-2026</t>
         </is>
       </c>
     </row>
@@ -59763,41 +59759,41 @@
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>GDC: The State of the Game Industry 2026</t>
+          <t>The state of video games with Matthew Ball – Part One</t>
         </is>
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Analysis</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr"/>
       <c r="E92" s="3" t="inlineStr">
         <is>
-          <t>https://gamedevreports.substack.com/p/gdc-the-state-of-the-game-industry-fcf</t>
+          <t>https://www.thegamebusiness.com/p/the-state-of-video-games-with-matthew</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>Platforms bet on exclusivity again</t>
+          <t>Studio investment in games plummets</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>Should PlayStation and Xbox change their plans on exclusive games?</t>
+          <t>GDC: The State of the Game Industry 2026</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>Analysis</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr"/>
       <c r="E93" s="3" t="inlineStr">
         <is>
-          <t>https://www.thegamebusiness.com/p/should-playstation-and-xbox-change</t>
+          <t>https://gamedevreports.substack.com/p/gdc-the-state-of-the-game-industry-fcf</t>
         </is>
       </c>
     </row>
@@ -59809,18 +59805,18 @@
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>Xbox console exclusives are returning on a ‘case-by-case’ basis</t>
+          <t>Should PlayStation and Xbox change their plans on exclusive games?</t>
         </is>
       </c>
       <c r="C94" s="3" t="inlineStr">
         <is>
-          <t>Reporting</t>
+          <t>Analysis</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr"/>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>https://www.gamedeveloper.com/business/xbox-console-exclusives-are-returning-on-a-case-by-case-basis</t>
+          <t>https://www.thegamebusiness.com/p/should-playstation-and-xbox-change</t>
         </is>
       </c>
     </row>
@@ -59832,7 +59828,7 @@
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>Xbox multiplayer and live service games will still be multiplatform, Matt Booty says</t>
+          <t>Xbox console exclusives are returning on a ‘case-by-case’ basis</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
@@ -59843,30 +59839,30 @@
       <c r="D95" s="3" t="inlineStr"/>
       <c r="E95" s="3" t="inlineStr">
         <is>
-          <t>https://www.videogameschronicle.com/news/xbox-multiplayer-and-live-service-games-will-still-be-multiplatform-going-forward-matt-booty-says/</t>
+          <t>https://www.gamedeveloper.com/business/xbox-console-exclusives-are-returning-on-a-case-by-case-basis</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="3" t="inlineStr">
         <is>
-          <t>Mobile has shifted from downloads to spending</t>
+          <t>Platforms bet on exclusivity again</t>
         </is>
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>State of Mobile 2026: 9 Key Trends</t>
+          <t>Xbox multiplayer and live service games will still be multiplatform, Matt Booty says</t>
         </is>
       </c>
       <c r="C96" s="3" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Reporting</t>
         </is>
       </c>
       <c r="D96" s="3" t="inlineStr"/>
       <c r="E96" s="3" t="inlineStr">
         <is>
-          <t>https://www.deconstructoroffun.com/blog/2026/2/2/state-of-mobile-2026</t>
+          <t>https://www.videogameschronicle.com/news/xbox-multiplayer-and-live-service-games-will-still-be-multiplatform-going-forward-matt-booty-says/</t>
         </is>
       </c>
     </row>
@@ -59878,18 +59874,18 @@
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>H1 2026: 4X Strategy's UA Reckoning</t>
+          <t>State of Mobile 2026: 9 Key Trends</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>Analysis</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="D97" s="3" t="inlineStr"/>
       <c r="E97" s="3" t="inlineStr">
         <is>
-          <t>https://naavik.co/f2p-mobile/h1-2026-4x-strategys-ua-reckoning/</t>
+          <t>https://www.deconstructoroffun.com/blog/2026/2/2/state-of-mobile-2026</t>
         </is>
       </c>
     </row>
@@ -59901,30 +59897,30 @@
       </c>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t>H1 2026 genre analysis: strategy stumbles, RPGs fall, and puzzle revenue ramps up</t>
+          <t>H1 2026: 4X Strategy's UA Reckoning</t>
         </is>
       </c>
       <c r="C98" s="3" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Analysis</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr"/>
       <c r="E98" s="3" t="inlineStr">
         <is>
-          <t>https://www.pocketgamer.biz/h1-2026-genre-analysis-strategy-stumbles-rpgs-fall-and-puzzle-revenue-ramps-up/</t>
+          <t>https://naavik.co/f2p-mobile/h1-2026-4x-strategys-ua-reckoning/</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
         <is>
-          <t>Creators are how players find games</t>
+          <t>Mobile has shifted from downloads to spending</t>
         </is>
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>GDC: The State of the Game Industry 2026</t>
+          <t>H1 2026 genre analysis: strategy stumbles, RPGs fall, and puzzle revenue ramps up</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
@@ -59935,7 +59931,7 @@
       <c r="D99" s="3" t="inlineStr"/>
       <c r="E99" s="3" t="inlineStr">
         <is>
-          <t>https://gamedevreports.substack.com/p/gdc-the-state-of-the-game-industry-fcf</t>
+          <t>https://www.pocketgamer.biz/h1-2026-genre-analysis-strategy-stumbles-rpgs-fall-and-puzzle-revenue-ramps-up/</t>
         </is>
       </c>
     </row>
@@ -59947,18 +59943,18 @@
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>14 trends for the next 5 years of PC/console games</t>
+          <t>GDC: The State of the Game Industry 2026</t>
         </is>
       </c>
       <c r="C100" s="3" t="inlineStr">
         <is>
-          <t>Analysis</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="D100" s="3" t="inlineStr"/>
       <c r="E100" s="3" t="inlineStr">
         <is>
-          <t>https://newsletter.gamediscover.co/p/14-trends-for-the-next-5-years-of</t>
+          <t>https://gamedevreports.substack.com/p/gdc-the-state-of-the-game-industry-fcf</t>
         </is>
       </c>
     </row>
@@ -59970,30 +59966,30 @@
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>H1 2026: 4X Strategy's UA Reckoning</t>
+          <t>14 trends for the next 5 years of PC/console games</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Analysis</t>
         </is>
       </c>
       <c r="D101" s="3" t="inlineStr"/>
       <c r="E101" s="3" t="inlineStr">
         <is>
-          <t>https://naavik.co/f2p-mobile/h1-2026-4x-strategys-ua-reckoning/</t>
+          <t>https://newsletter.gamediscover.co/p/14-trends-for-the-next-5-years-of</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="3" t="inlineStr">
         <is>
-          <t>New games fight for playtime</t>
+          <t>Creators are how players find games</t>
         </is>
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>Newzoo: PC and Console Market in 2026</t>
+          <t>H1 2026: 4X Strategy's UA Reckoning</t>
         </is>
       </c>
       <c r="C102" s="3" t="inlineStr">
@@ -60004,7 +60000,7 @@
       <c r="D102" s="3" t="inlineStr"/>
       <c r="E102" s="3" t="inlineStr">
         <is>
-          <t>https://gamedevreports.substack.com/p/newzoo-pc-and-console-market-in-2026</t>
+          <t>https://naavik.co/f2p-mobile/h1-2026-4x-strategys-ua-reckoning/</t>
         </is>
       </c>
     </row>
@@ -60016,18 +60012,18 @@
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>Why older games rule – and new games drool – in Discoveryland</t>
+          <t>Newzoo: PC and Console Market in 2026</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
         <is>
-          <t>Analysis</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="D103" s="3" t="inlineStr"/>
       <c r="E103" s="3" t="inlineStr">
         <is>
-          <t>https://newsletter.gamediscover.co/p/why-older-games-rule-and-new-games</t>
+          <t>https://gamedevreports.substack.com/p/newzoo-pc-and-console-market-in-2026</t>
         </is>
       </c>
     </row>
@@ -60039,41 +60035,41 @@
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>Steam users spent only 15% of their time on games released in 2024</t>
+          <t>Why older games rule – and new games drool – in Discoveryland</t>
         </is>
       </c>
       <c r="C104" s="3" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Analysis</t>
         </is>
       </c>
       <c r="D104" s="3" t="inlineStr"/>
       <c r="E104" s="3" t="inlineStr">
         <is>
-          <t>https://gamedevreports.substack.com/p/steam-users-spent-only-15-of-their</t>
+          <t>https://newsletter.gamediscover.co/p/why-older-games-rule-and-new-games</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="3" t="inlineStr">
         <is>
-          <t>The rise of friendslop</t>
+          <t>New games fight for playtime</t>
         </is>
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>GameDiscoverCo: Most successful new releases on PC and Consoles in 2025</t>
+          <t>Valve has reportedly made £11bn from Steam already in 2026, and biggest earning new arrival is Forza Horizon 6</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Reporting</t>
         </is>
       </c>
       <c r="D105" s="3" t="inlineStr"/>
       <c r="E105" s="3" t="inlineStr">
         <is>
-          <t>https://gamedevreports.substack.com/p/gamediscoverco-most-successful-new</t>
+          <t>https://www.eurogamer.net/forza-horizon-6-biggest-steam-new-release-11-billion-gbp</t>
         </is>
       </c>
     </row>
@@ -60085,18 +60081,18 @@
       </c>
       <c r="B106" s="3" t="inlineStr">
         <is>
-          <t>What developers can learn from indie social co-op</t>
+          <t>GameDiscoverCo: Most successful new releases on PC and Consoles in 2025</t>
         </is>
       </c>
       <c r="C106" s="3" t="inlineStr">
         <is>
-          <t>Analysis</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="D106" s="3" t="inlineStr"/>
       <c r="E106" s="3" t="inlineStr">
         <is>
-          <t>https://www.gamedeveloper.com/design/what-developers-can-learn-from-the-indie-social-co-op-games-topping-the-steam-charts</t>
+          <t>https://gamedevreports.substack.com/p/gamediscoverco-most-successful-new</t>
         </is>
       </c>
     </row>
@@ -60108,41 +60104,41 @@
       </c>
       <c r="B107" s="3" t="inlineStr">
         <is>
-          <t>Calling games like Peak and REPO ‘friendslop’ devalues the developer, investor says</t>
+          <t>What developers can learn from indie social co-op</t>
         </is>
       </c>
       <c r="C107" s="3" t="inlineStr">
         <is>
-          <t>Reporting</t>
+          <t>Analysis</t>
         </is>
       </c>
       <c r="D107" s="3" t="inlineStr"/>
       <c r="E107" s="3" t="inlineStr">
         <is>
-          <t>https://www.gamesradar.com/games/co-op/calling-steam-games-like-peak-and-repo-friendslop-devalues-the-skill-of-the-developer-industry-investor-says-so-lets-collectively-kill-the-term-before-its-too-late/</t>
+          <t>https://www.gamedeveloper.com/design/what-developers-can-learn-from-the-indie-social-co-op-games-topping-the-steam-charts</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="3" t="inlineStr">
         <is>
-          <t>Live ops is becoming a playbook</t>
+          <t>The rise of friendslop</t>
         </is>
       </c>
       <c r="B108" s="3" t="inlineStr">
         <is>
-          <t>Converging Live Ops Trends in Mobile Puzzle</t>
+          <t>Calling games like Peak and REPO ‘friendslop’ devalues the developer, investor says</t>
         </is>
       </c>
       <c r="C108" s="3" t="inlineStr">
         <is>
-          <t>Analysis</t>
+          <t>Reporting</t>
         </is>
       </c>
       <c r="D108" s="3" t="inlineStr"/>
       <c r="E108" s="3" t="inlineStr">
         <is>
-          <t>https://naavik.co/digest/live-ops-trends-powering-mobile-puzzle/</t>
+          <t>https://www.gamesradar.com/games/co-op/calling-steam-games-like-peak-and-repo-friendslop-devalues-the-skill-of-the-developer-industry-investor-says-so-lets-collectively-kill-the-term-before-its-too-late/</t>
         </is>
       </c>
     </row>
@@ -60154,18 +60150,18 @@
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>H1 2026: 4X Strategy's UA Reckoning</t>
+          <t>Converging Live Ops Trends in Mobile Puzzle</t>
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Analysis</t>
         </is>
       </c>
       <c r="D109" s="3" t="inlineStr"/>
       <c r="E109" s="3" t="inlineStr">
         <is>
-          <t>https://naavik.co/f2p-mobile/h1-2026-4x-strategys-ua-reckoning/</t>
+          <t>https://naavik.co/digest/live-ops-trends-powering-mobile-puzzle/</t>
         </is>
       </c>
     </row>
@@ -60177,23 +60173,46 @@
       </c>
       <c r="B110" s="3" t="inlineStr">
         <is>
-          <t>Book Excerpt: Running a Successful Live Service Game</t>
+          <t>H1 2026: 4X Strategy's UA Reckoning</t>
         </is>
       </c>
       <c r="C110" s="3" t="inlineStr">
         <is>
-          <t>Analysis</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="D110" s="3" t="inlineStr"/>
       <c r="E110" s="3" t="inlineStr">
         <is>
+          <t>https://naavik.co/f2p-mobile/h1-2026-4x-strategys-ua-reckoning/</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="3" t="inlineStr">
+        <is>
+          <t>Live ops is becoming a playbook</t>
+        </is>
+      </c>
+      <c r="B111" s="3" t="inlineStr">
+        <is>
+          <t>Book Excerpt: Running a Successful Live Service Game</t>
+        </is>
+      </c>
+      <c r="C111" s="3" t="inlineStr">
+        <is>
+          <t>Analysis</t>
+        </is>
+      </c>
+      <c r="D111" s="3" t="inlineStr"/>
+      <c r="E111" s="3" t="inlineStr">
+        <is>
           <t>https://www.gamedeveloper.com/business/book-excerpt-running-a-successful-live-service-game</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E110"/>
+  <autoFilter ref="A1:E111"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update the data to the workbook of 2026-09-11
914 sources, 10 markets, 37 trends, 35 platforms, 30 genres.

Copied from public/downloads/ by scripts/build-mirror.mjs in the site
repository. Every count in the README is read from data/downloads.json rather
than typed, so it describes the files beside it.
</commit_message>
<xml_diff>
--- a/games-research-starter-pack.xlsx
+++ b/games-research-starter-pack.xlsx
@@ -18,7 +18,7 @@
     <sheet name="Vocabulary" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sources'!$A$1:$R$888</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sources'!$A$1:$R$915</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Trends'!$A$1:$H$38</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Trend reading'!$A$1:$E$111</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Platforms'!$A$1:$F$36</definedName>
@@ -474,7 +474,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Compiled from the research workbook of 2026-09-10. https://games.thisisdelightful.com</t>
+          <t>Compiled from the research workbook of 2026-09-11. https://games.thisisdelightful.com</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>887</v>
+        <v>914</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -640,7 +640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R888"/>
+  <dimension ref="A1:R915"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -54366,12 +54366,12 @@
     <row r="862">
       <c r="A862" s="3" t="inlineStr">
         <is>
-          <t>r-zocken</t>
+          <t>r-gaming</t>
         </is>
       </c>
       <c r="B862" s="3" t="inlineStr">
         <is>
-          <t>r/zocken</t>
+          <t>r/gaming</t>
         </is>
       </c>
       <c r="C862" s="3" t="inlineStr">
@@ -54391,17 +54391,17 @@
       </c>
       <c r="F862" s="3" t="inlineStr">
         <is>
-          <t>General German-language player sentiment and discussion. The venue for German community temperature on Reddit, not r/de. Never for citation. The main German-language gaming community.</t>
+          <t>The mass-market front page of gaming on Reddit and the largest games community anywhere, tens of millions strong. Memes, screenshots and outrage rather than discussion, which is what makes it a temperature read: what reaches its front page is what the general player has noticed.</t>
         </is>
       </c>
       <c r="G862" s="3" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>US</t>
         </is>
       </c>
       <c r="H862" s="3" t="inlineStr">
         <is>
-          <t>German</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I862" s="3" t="inlineStr">
@@ -54411,7 +54411,7 @@
       </c>
       <c r="J862" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/zocken</t>
+          <t>https://www.reddit.com/r/gaming/</t>
         </is>
       </c>
       <c r="K862" s="3" t="inlineStr"/>
@@ -54426,12 +54426,12 @@
     <row r="863">
       <c r="A863" s="3" t="inlineStr">
         <is>
-          <t>r-pcgamingde</t>
+          <t>r-games</t>
         </is>
       </c>
       <c r="B863" s="3" t="inlineStr">
         <is>
-          <t>r/PCGamingDE</t>
+          <t>r/Games</t>
         </is>
       </c>
       <c r="C863" s="3" t="inlineStr">
@@ -54451,17 +54451,17 @@
       </c>
       <c r="F863" s="3" t="inlineStr">
         <is>
-          <t>German-language PC gaming discussion, builds, and platform sentiment.</t>
+          <t>The moderated news-and-discussion sub, where an industry story gets its first large English-language comment thread. Nearer the trade conversation than r/gaming and the better read of informed player reaction to layoffs, pricing and platform moves.</t>
         </is>
       </c>
       <c r="G863" s="3" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>US</t>
         </is>
       </c>
       <c r="H863" s="3" t="inlineStr">
         <is>
-          <t>German</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I863" s="3" t="inlineStr">
@@ -54471,7 +54471,7 @@
       </c>
       <c r="J863" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/PCGamingDE</t>
+          <t>https://www.reddit.com/r/Games/</t>
         </is>
       </c>
       <c r="K863" s="3" t="inlineStr"/>
@@ -54486,12 +54486,12 @@
     <row r="864">
       <c r="A864" s="3" t="inlineStr">
         <is>
-          <t>r-jeuxvideo</t>
+          <t>r-truegaming</t>
         </is>
       </c>
       <c r="B864" s="3" t="inlineStr">
         <is>
-          <t>r/jeuxvideo</t>
+          <t>r/truegaming</t>
         </is>
       </c>
       <c r="C864" s="3" t="inlineStr">
@@ -54511,17 +54511,17 @@
       </c>
       <c r="F864" s="3" t="inlineStr">
         <is>
-          <t>The main French-language gaming community. French player sentiment and discussion at scale, including esports threads. Not affiliated with the Webedia site jeuxvideo.com despite the shared name.</t>
+          <t>Long-form argument about design, culture and the industry, with memes and news banned. Where a discourse gets worked out at length rather than reacted to.</t>
         </is>
       </c>
       <c r="G864" s="3" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>US</t>
         </is>
       </c>
       <c r="H864" s="3" t="inlineStr">
         <is>
-          <t>French</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I864" s="3" t="inlineStr">
@@ -54531,7 +54531,7 @@
       </c>
       <c r="J864" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/jeuxvideo</t>
+          <t>https://www.reddit.com/r/truegaming/</t>
         </is>
       </c>
       <c r="K864" s="3" t="inlineStr"/>
@@ -54546,12 +54546,12 @@
     <row r="865">
       <c r="A865" s="3" t="inlineStr">
         <is>
-          <t>r-italygames</t>
+          <t>r-patientgamers</t>
         </is>
       </c>
       <c r="B865" s="3" t="inlineStr">
         <is>
-          <t>r/italygames</t>
+          <t>r/patientgamers</t>
         </is>
       </c>
       <c r="C865" s="3" t="inlineStr">
@@ -54571,17 +54571,17 @@
       </c>
       <c r="F865" s="3" t="inlineStr">
         <is>
-          <t>Italian player sentiment across PC, console, retro, and tabletop. The venue for Italian community temperature on Reddit, not r/italy. The main Italian gaming community.</t>
+          <t>Players who wait a year or more before buying. The backlog, price-sensitivity and anti-hype cohort in its own words, and a counterweight to the launch-week sentiment everywhere else.</t>
         </is>
       </c>
       <c r="G865" s="3" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>US</t>
         </is>
       </c>
       <c r="H865" s="3" t="inlineStr">
         <is>
-          <t>Italian</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I865" s="3" t="inlineStr">
@@ -54591,7 +54591,7 @@
       </c>
       <c r="J865" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/italygames</t>
+          <t>https://www.reddit.com/r/patientgamers/</t>
         </is>
       </c>
       <c r="K865" s="3" t="inlineStr"/>
@@ -54606,12 +54606,12 @@
     <row r="866">
       <c r="A866" s="3" t="inlineStr">
         <is>
-          <t>r-gamedevelopersitaly</t>
+          <t>r-pcgaming</t>
         </is>
       </c>
       <c r="B866" s="3" t="inlineStr">
         <is>
-          <t>r/GameDevelopersItaly</t>
+          <t>r/pcgaming</t>
         </is>
       </c>
       <c r="C866" s="3" t="inlineStr">
@@ -54631,17 +54631,17 @@
       </c>
       <c r="F866" s="3" t="inlineStr">
         <is>
-          <t>Italian-language developer discussion. Useful as a window on the Italian dev scene, which has no trade press.</t>
+          <t>PC platform news and sentiment: launchers, DRM, anti-cheat, ports, Game Pass and storefront pricing. Where the PC side of a platform argument is made.</t>
         </is>
       </c>
       <c r="G866" s="3" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>US</t>
         </is>
       </c>
       <c r="H866" s="3" t="inlineStr">
         <is>
-          <t>Italian</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I866" s="3" t="inlineStr">
@@ -54651,7 +54651,7 @@
       </c>
       <c r="J866" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/GameDevelopersItaly</t>
+          <t>https://www.reddit.com/r/pcgaming/</t>
         </is>
       </c>
       <c r="K866" s="3" t="inlineStr"/>
@@ -54666,12 +54666,12 @@
     <row r="867">
       <c r="A867" s="3" t="inlineStr">
         <is>
-          <t>r-gamesecultura</t>
+          <t>r-nintendoswitch</t>
         </is>
       </c>
       <c r="B867" s="3" t="inlineStr">
         <is>
-          <t>r/gamesEcultura</t>
+          <t>r/NintendoSwitch</t>
         </is>
       </c>
       <c r="C867" s="3" t="inlineStr">
@@ -54691,17 +54691,17 @@
       </c>
       <c r="F867" s="3" t="inlineStr">
         <is>
-          <t>Brazilian player sentiment where games meet wider geek culture. The biggest Reddit venue for Brazilian community temperature. The largest Brazilian gaming community.</t>
+          <t>The Nintendo platform community through the Switch 2 transition. Family and handheld play, hardware and game pricing, and first-party release reaction.</t>
         </is>
       </c>
       <c r="G867" s="3" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>US</t>
         </is>
       </c>
       <c r="H867" s="3" t="inlineStr">
         <is>
-          <t>Portuguese</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I867" s="3" t="inlineStr">
@@ -54711,7 +54711,7 @@
       </c>
       <c r="J867" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/gamesEcultura</t>
+          <t>https://www.reddit.com/r/NintendoSwitch/</t>
         </is>
       </c>
       <c r="K867" s="3" t="inlineStr"/>
@@ -54726,12 +54726,12 @@
     <row r="868">
       <c r="A868" s="3" t="inlineStr">
         <is>
-          <t>r-jogosbrasil</t>
+          <t>r-ps5</t>
         </is>
       </c>
       <c r="B868" s="3" t="inlineStr">
         <is>
-          <t>r/jogosbrasil</t>
+          <t>r/PS5</t>
         </is>
       </c>
       <c r="C868" s="3" t="inlineStr">
@@ -54751,17 +54751,17 @@
       </c>
       <c r="F868" s="3" t="inlineStr">
         <is>
-          <t>Brazilian discussion of PC, console, and mobile games plus release and free-game news.</t>
+          <t>PlayStation platform sentiment on exclusives, PS Plus tiers and hardware pricing.</t>
         </is>
       </c>
       <c r="G868" s="3" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>US</t>
         </is>
       </c>
       <c r="H868" s="3" t="inlineStr">
         <is>
-          <t>Portuguese</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I868" s="3" t="inlineStr">
@@ -54771,7 +54771,7 @@
       </c>
       <c r="J868" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/jogosbrasil</t>
+          <t>https://www.reddit.com/r/PS5/</t>
         </is>
       </c>
       <c r="K868" s="3" t="inlineStr"/>
@@ -54786,12 +54786,12 @@
     <row r="869">
       <c r="A869" s="3" t="inlineStr">
         <is>
-          <t>r-playstationbrasil</t>
+          <t>r-xbox</t>
         </is>
       </c>
       <c r="B869" s="3" t="inlineStr">
         <is>
-          <t>r/playstationbrasil</t>
+          <t>r/xbox</t>
         </is>
       </c>
       <c r="C869" s="3" t="inlineStr">
@@ -54811,17 +54811,17 @@
       </c>
       <c r="F869" s="3" t="inlineStr">
         <is>
-          <t>Brazilian platform-specific sentiment, pricing complaints, and buying culture on PlayStation.</t>
+          <t>Xbox platform sentiment, with Game Pass value and the shift to multiplatform releases as its running arguments. r/XboxSeriesX went quiet in mid-2024 and points here.</t>
         </is>
       </c>
       <c r="G869" s="3" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>US</t>
         </is>
       </c>
       <c r="H869" s="3" t="inlineStr">
         <is>
-          <t>Portuguese</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I869" s="3" t="inlineStr">
@@ -54831,7 +54831,7 @@
       </c>
       <c r="J869" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/playstationbrasil</t>
+          <t>https://www.reddit.com/r/xbox/</t>
         </is>
       </c>
       <c r="K869" s="3" t="inlineStr"/>
@@ -54846,12 +54846,12 @@
     <row r="870">
       <c r="A870" s="3" t="inlineStr">
         <is>
-          <t>r-jogatina</t>
+          <t>r-steamdeck</t>
         </is>
       </c>
       <c r="B870" s="3" t="inlineStr">
         <is>
-          <t>r/jogatina</t>
+          <t>r/SteamDeck</t>
         </is>
       </c>
       <c r="C870" s="3" t="inlineStr">
@@ -54871,17 +54871,17 @@
       </c>
       <c r="F870" s="3" t="inlineStr">
         <is>
-          <t>Brazilian general games discussion.</t>
+          <t>The handheld PC resurgence from the owner side: what runs, what gets bought, and the Deck Verified purchase habit. Unusually fast growth for a hardware sub.</t>
         </is>
       </c>
       <c r="G870" s="3" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>US</t>
         </is>
       </c>
       <c r="H870" s="3" t="inlineStr">
         <is>
-          <t>Portuguese</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I870" s="3" t="inlineStr">
@@ -54891,7 +54891,7 @@
       </c>
       <c r="J870" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/jogatina</t>
+          <t>https://www.reddit.com/r/SteamDeck/</t>
         </is>
       </c>
       <c r="K870" s="3" t="inlineStr"/>
@@ -54906,12 +54906,12 @@
     <row r="871">
       <c r="A871" s="3" t="inlineStr">
         <is>
-          <t>r-videojuegosmx</t>
+          <t>r-minecraft</t>
         </is>
       </c>
       <c r="B871" s="3" t="inlineStr">
         <is>
-          <t>r/VideojuegosMX</t>
+          <t>r/Minecraft</t>
         </is>
       </c>
       <c r="C871" s="3" t="inlineStr">
@@ -54931,17 +54931,17 @@
       </c>
       <c r="F871" s="3" t="inlineStr">
         <is>
-          <t>Mexican player sentiment and discussion.</t>
+          <t>The largest sandbox community, mixing builds, children's first posts and parents asking about editions and servers. The lived side of the sandbox and UGC story.</t>
         </is>
       </c>
       <c r="G871" s="3" t="inlineStr">
         <is>
-          <t>MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="H871" s="3" t="inlineStr">
         <is>
-          <t>Spanish</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I871" s="3" t="inlineStr">
@@ -54951,7 +54951,7 @@
       </c>
       <c r="J871" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/VideojuegosMX</t>
+          <t>https://www.reddit.com/r/Minecraft/</t>
         </is>
       </c>
       <c r="K871" s="3" t="inlineStr"/>
@@ -54966,12 +54966,12 @@
     <row r="872">
       <c r="A872" s="3" t="inlineStr">
         <is>
-          <t>r-videojuegos</t>
+          <t>r-roblox</t>
         </is>
       </c>
       <c r="B872" s="3" t="inlineStr">
         <is>
-          <t>r/videojuegos</t>
+          <t>r/roblox</t>
         </is>
       </c>
       <c r="C872" s="3" t="inlineStr">
@@ -54991,17 +54991,17 @@
       </c>
       <c r="F872" s="3" t="inlineStr">
         <is>
-          <t>Spanish-language player sentiment across Spain and Latin America. A language venue rather than a country venue, so read alongside the national subs.</t>
+          <t>Unofficial, and unhappy with the platform as often as not: creator payouts, moderation, age checks and parents asking what their child is actually playing. Read alongside r/Parenting.</t>
         </is>
       </c>
       <c r="G872" s="3" t="inlineStr">
         <is>
-          <t>ES; LATAM; MX</t>
+          <t>US</t>
         </is>
       </c>
       <c r="H872" s="3" t="inlineStr">
         <is>
-          <t>Spanish</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I872" s="3" t="inlineStr">
@@ -55011,7 +55011,7 @@
       </c>
       <c r="J872" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/videojuegos/</t>
+          <t>https://www.reddit.com/r/roblox/</t>
         </is>
       </c>
       <c r="K872" s="3" t="inlineStr"/>
@@ -55026,12 +55026,12 @@
     <row r="873">
       <c r="A873" s="3" t="inlineStr">
         <is>
-          <t>r-esgaming</t>
+          <t>r-fortnitebr</t>
         </is>
       </c>
       <c r="B873" s="3" t="inlineStr">
         <is>
-          <t>r/esGaming</t>
+          <t>r/FortNiteBR</t>
         </is>
       </c>
       <c r="C873" s="3" t="inlineStr">
@@ -55051,17 +55051,17 @@
       </c>
       <c r="F873" s="3" t="inlineStr">
         <is>
-          <t>Spanish player sentiment and discussion at scale. Sits alongside the Mediavida forum rather than replacing it.</t>
+          <t>The Fortnite community, run with developer support, so patch, item-shop and collaboration reaction lands here first. Younger than r/Games and the place to read creator-map and UGC sentiment.</t>
         </is>
       </c>
       <c r="G873" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>US</t>
         </is>
       </c>
       <c r="H873" s="3" t="inlineStr">
         <is>
-          <t>Spanish</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I873" s="3" t="inlineStr">
@@ -55071,7 +55071,7 @@
       </c>
       <c r="J873" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/esGaming</t>
+          <t>https://www.reddit.com/r/FortNiteBR/</t>
         </is>
       </c>
       <c r="K873" s="3" t="inlineStr"/>
@@ -55086,12 +55086,12 @@
     <row r="874">
       <c r="A874" s="3" t="inlineStr">
         <is>
-          <t>r-geymingtr</t>
+          <t>r-parenting</t>
         </is>
       </c>
       <c r="B874" s="3" t="inlineStr">
         <is>
-          <t>r/GeymingTr</t>
+          <t>r/Parenting</t>
         </is>
       </c>
       <c r="C874" s="3" t="inlineStr">
@@ -55111,17 +55111,17 @@
       </c>
       <c r="F874" s="3" t="inlineStr">
         <is>
-          <t>Turkish player sentiment in a casual register. The name is a phonetic spelling of gaming, an instance of the English loanword doing the work the betting-polluted word oyun cannot.</t>
+          <t>Not a games sub, and that is the point: screen time, Roblox safety and Fortnite arguments as parents who do not play describe them. Search it for a game's name rather than browsing it.</t>
         </is>
       </c>
       <c r="G874" s="3" t="inlineStr">
         <is>
-          <t>TR</t>
+          <t>US</t>
         </is>
       </c>
       <c r="H874" s="3" t="inlineStr">
         <is>
-          <t>Turkish</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I874" s="3" t="inlineStr">
@@ -55131,7 +55131,7 @@
       </c>
       <c r="J874" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/GeymingTr</t>
+          <t>https://www.reddit.com/r/Parenting/</t>
         </is>
       </c>
       <c r="K874" s="3" t="inlineStr"/>
@@ -55146,12 +55146,12 @@
     <row r="875">
       <c r="A875" s="3" t="inlineStr">
         <is>
-          <t>r-oyun</t>
+          <t>r-daddit</t>
         </is>
       </c>
       <c r="B875" s="3" t="inlineStr">
         <is>
-          <t>r/oyun</t>
+          <t>r/daddit</t>
         </is>
       </c>
       <c r="C875" s="3" t="inlineStr">
@@ -55171,17 +55171,17 @@
       </c>
       <c r="F875" s="3" t="inlineStr">
         <is>
-          <t>Turkish general games discussion, the second general venue alongside r/GeymingTr.</t>
+          <t>Fathers, a great many of them players, on co-play, first consoles, screen-time rules and what to let a child play. The nearest thing to a gamer-parents venue at scale.</t>
         </is>
       </c>
       <c r="G875" s="3" t="inlineStr">
         <is>
-          <t>TR</t>
+          <t>US</t>
         </is>
       </c>
       <c r="H875" s="3" t="inlineStr">
         <is>
-          <t>Turkish</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I875" s="3" t="inlineStr">
@@ -55191,7 +55191,7 @@
       </c>
       <c r="J875" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/oyun</t>
+          <t>https://www.reddit.com/r/daddit/</t>
         </is>
       </c>
       <c r="K875" s="3" t="inlineStr"/>
@@ -55206,12 +55206,12 @@
     <row r="876">
       <c r="A876" s="3" t="inlineStr">
         <is>
-          <t>r-trgamedeveloper</t>
+          <t>r-gamedev</t>
         </is>
       </c>
       <c r="B876" s="3" t="inlineStr">
         <is>
-          <t>r/TrGameDeveloper</t>
+          <t>r/gamedev</t>
         </is>
       </c>
       <c r="C876" s="3" t="inlineStr">
@@ -55231,17 +55231,17 @@
       </c>
       <c r="F876" s="3" t="inlineStr">
         <is>
-          <t>Turkish developer discussion and publishing help. The largest gamedev subreddit found, consistent with Turkey's production-market profile.</t>
+          <t>The largest developer community, so the layoff era, publishing terms, Steam visibility and AI-in-development arguments appear here from the maker's side. Small-studio and hobbyist voices dominate.</t>
         </is>
       </c>
       <c r="G876" s="3" t="inlineStr">
         <is>
-          <t>TR</t>
+          <t>US</t>
         </is>
       </c>
       <c r="H876" s="3" t="inlineStr">
         <is>
-          <t>Turkish</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I876" s="3" t="inlineStr">
@@ -55251,7 +55251,7 @@
       </c>
       <c r="J876" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/TrGameDeveloper</t>
+          <t>https://www.reddit.com/r/gamedev/</t>
         </is>
       </c>
       <c r="K876" s="3" t="inlineStr"/>
@@ -55266,12 +55266,12 @@
     <row r="877">
       <c r="A877" s="3" t="inlineStr">
         <is>
-          <t>r-turkoyunsektoru</t>
+          <t>r-gamingleaksandrumours</t>
         </is>
       </c>
       <c r="B877" s="3" t="inlineStr">
         <is>
-          <t>r/TurkOyunSektoru</t>
+          <t>r/GamingLeaksAndRumours</t>
         </is>
       </c>
       <c r="C877" s="3" t="inlineStr">
@@ -55291,17 +55291,17 @@
       </c>
       <c r="F877" s="3" t="inlineStr">
         <is>
-          <t>Turkish industry and publishing discussion, the business side of the scene r/TrGameDeveloper covers from the craft side.</t>
+          <t>Where leaks and rumours are gathered and argued over before an announcement. Useful for tracing when a story broke and how it was received, never for what is true.</t>
         </is>
       </c>
       <c r="G877" s="3" t="inlineStr">
         <is>
-          <t>TR</t>
+          <t>US</t>
         </is>
       </c>
       <c r="H877" s="3" t="inlineStr">
         <is>
-          <t>Turkish</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I877" s="3" t="inlineStr">
@@ -55311,7 +55311,7 @@
       </c>
       <c r="J877" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/TurkOyunSektoru</t>
+          <t>https://www.reddit.com/r/GamingLeaksAndRumours/</t>
         </is>
       </c>
       <c r="K877" s="3" t="inlineStr"/>
@@ -55326,12 +55326,12 @@
     <row r="878">
       <c r="A878" s="3" t="inlineStr">
         <is>
-          <t>r-saudi-gamers</t>
+          <t>r-gachagaming</t>
         </is>
       </c>
       <c r="B878" s="3" t="inlineStr">
         <is>
-          <t>r/saudi_gamers</t>
+          <t>r/gachagaming</t>
         </is>
       </c>
       <c r="C878" s="3" t="inlineStr">
@@ -55351,17 +55351,17 @@
       </c>
       <c r="F878" s="3" t="inlineStr">
         <is>
-          <t>Saudi and pan-Arab player sentiment. One of the few venues in the MENA stack with no institutional or state-linked owner.</t>
+          <t>Gacha and live-service mobile discourse: monetization, banners, revenue-chart threads and end-of-service watches. The best English read on the Asian mobile model as US players experience it.</t>
         </is>
       </c>
       <c r="G878" s="3" t="inlineStr">
         <is>
-          <t>MENA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="H878" s="3" t="inlineStr">
         <is>
-          <t>Arabic</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I878" s="3" t="inlineStr">
@@ -55371,7 +55371,7 @@
       </c>
       <c r="J878" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/saudi_gamers</t>
+          <t>https://www.reddit.com/r/gachagaming/</t>
         </is>
       </c>
       <c r="K878" s="3" t="inlineStr"/>
@@ -55386,12 +55386,12 @@
     <row r="879">
       <c r="A879" s="3" t="inlineStr">
         <is>
-          <t>r-iraqigamers</t>
+          <t>r-androidgaming-and-r-iosgaming</t>
         </is>
       </c>
       <c r="B879" s="3" t="inlineStr">
         <is>
-          <t>r/Iraqigamers</t>
+          <t>r/AndroidGaming and r/iosgaming</t>
         </is>
       </c>
       <c r="C879" s="3" t="inlineStr">
@@ -55411,17 +55411,17 @@
       </c>
       <c r="F879" s="3" t="inlineStr">
         <is>
-          <t>Iraqi player sentiment and memes.</t>
+          <t>Mobile gaming from the player side, one sub per store, with premium and ad-free titles favoured over free-to-play in both. Where the app-store unbundling and mobile spending trends meet the people paying.</t>
         </is>
       </c>
       <c r="G879" s="3" t="inlineStr">
         <is>
-          <t>MENA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="H879" s="3" t="inlineStr">
         <is>
-          <t>Arabic</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I879" s="3" t="inlineStr">
@@ -55431,7 +55431,7 @@
       </c>
       <c r="J879" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/Iraqigamers</t>
+          <t>https://www.reddit.com/r/AndroidGaming/</t>
         </is>
       </c>
       <c r="K879" s="3" t="inlineStr"/>
@@ -55446,12 +55446,12 @@
     <row r="880">
       <c r="A880" s="3" t="inlineStr">
         <is>
-          <t>r-egyptgaming-and-r-egyptgamingg</t>
+          <t>r-esports</t>
         </is>
       </c>
       <c r="B880" s="3" t="inlineStr">
         <is>
-          <t>r/EgyptGaming and r/EgyptGaminGG</t>
+          <t>r/esports</t>
         </is>
       </c>
       <c r="C880" s="3" t="inlineStr">
@@ -55471,17 +55471,17 @@
       </c>
       <c r="F880" s="3" t="inlineStr">
         <is>
-          <t>Egyptian player sentiment across two communities of similar size. Neither is clearly primary from outside, so both are listed.</t>
+          <t>Cross-title esports news and business: team finances, viewership, Gulf-backed events and the post-reckoning contraction. Title subs carry the fandom; this one carries the industry.</t>
         </is>
       </c>
       <c r="G880" s="3" t="inlineStr">
         <is>
-          <t>MENA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="H880" s="3" t="inlineStr">
         <is>
-          <t>Arabic</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I880" s="3" t="inlineStr">
@@ -55491,7 +55491,7 @@
       </c>
       <c r="J880" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/EgyptGaming</t>
+          <t>https://www.reddit.com/r/esports/</t>
         </is>
       </c>
       <c r="K880" s="3" t="inlineStr"/>
@@ -55506,12 +55506,12 @@
     <row r="881">
       <c r="A881" s="3" t="inlineStr">
         <is>
-          <t>r-arabic-games</t>
+          <t>r-gamedeals</t>
         </is>
       </c>
       <c r="B881" s="3" t="inlineStr">
         <is>
-          <t>r/Arabic_Games</t>
+          <t>r/GameDeals</t>
         </is>
       </c>
       <c r="C881" s="3" t="inlineStr">
@@ -55531,17 +55531,17 @@
       </c>
       <c r="F881" s="3" t="inlineStr">
         <is>
-          <t>Arabic localization discourse, official and fan translations. Small but the only localization venue in this directory.</t>
+          <t>Discounts and bundles posted as they appear. A live read on price sensitivity, the premium price ceiling and which storefronts players actually buy from.</t>
         </is>
       </c>
       <c r="G881" s="3" t="inlineStr">
         <is>
-          <t>MENA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="H881" s="3" t="inlineStr">
         <is>
-          <t>Arabic</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I881" s="3" t="inlineStr">
@@ -55551,7 +55551,7 @@
       </c>
       <c r="J881" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/Arabic_Games</t>
+          <t>https://www.reddit.com/r/GameDeals/</t>
         </is>
       </c>
       <c r="K881" s="3" t="inlineStr"/>
@@ -55566,12 +55566,12 @@
     <row r="882">
       <c r="A882" s="3" t="inlineStr">
         <is>
-          <t>r-spel</t>
+          <t>r-girlgamers</t>
         </is>
       </c>
       <c r="B882" s="3" t="inlineStr">
         <is>
-          <t>r/Spel</t>
+          <t>r/GirlGamers</t>
         </is>
       </c>
       <c r="C882" s="3" t="inlineStr">
@@ -55591,17 +55591,17 @@
       </c>
       <c r="F882" s="3" t="inlineStr">
         <is>
-          <t>Swedish player sentiment, the one national-language venue in a bloc that otherwise uses English subreddits. The name reclaims the word spel, which in Swedish search otherwise pulls betting companies first.</t>
+          <t>Women who play, on games, harassment and representation. One of the few large venues where the gaming culture war is discussed by its targets rather than its combatants.</t>
         </is>
       </c>
       <c r="G882" s="3" t="inlineStr">
         <is>
-          <t>Nordics</t>
+          <t>US</t>
         </is>
       </c>
       <c r="H882" s="3" t="inlineStr">
         <is>
-          <t>Swedish</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I882" s="3" t="inlineStr">
@@ -55611,7 +55611,7 @@
       </c>
       <c r="J882" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/Spel</t>
+          <t>https://www.reddit.com/r/GirlGamers/</t>
         </is>
       </c>
       <c r="K882" s="3" t="inlineStr"/>
@@ -55626,12 +55626,12 @@
     <row r="883">
       <c r="A883" s="3" t="inlineStr">
         <is>
-          <t>dutch-gaming-reddit</t>
+          <t>r-disabledgamers</t>
         </is>
       </c>
       <c r="B883" s="3" t="inlineStr">
         <is>
-          <t>Dutch gaming Reddit (r/GamingNL)</t>
+          <t>r/disabledgamers</t>
         </is>
       </c>
       <c r="C883" s="3" t="inlineStr">
@@ -55651,17 +55651,17 @@
       </c>
       <c r="F883" s="3" t="inlineStr">
         <is>
-          <t>Dutch gamers use the international English subreddits, and the national sub r/GamingNL stays around 1.5K members in a country of 18 million.</t>
+          <t>Accessibility from the player side: controllers, one-handed play, and which games can be played at all. Small, but the only accessibility venue in this directory.</t>
         </is>
       </c>
       <c r="G883" s="3" t="inlineStr">
         <is>
-          <t>NL</t>
+          <t>US</t>
         </is>
       </c>
       <c r="H883" s="3" t="inlineStr">
         <is>
-          <t>Dutch; English</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I883" s="3" t="inlineStr">
@@ -55671,7 +55671,7 @@
       </c>
       <c r="J883" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/GamingNL</t>
+          <t>https://www.reddit.com/r/disabledgamers/</t>
         </is>
       </c>
       <c r="K883" s="3" t="inlineStr"/>
@@ -55686,12 +55686,12 @@
     <row r="884">
       <c r="A884" s="3" t="inlineStr">
         <is>
-          <t>r-phgamers</t>
+          <t>r-stopgaming</t>
         </is>
       </c>
       <c r="B884" s="3" t="inlineStr">
         <is>
-          <t>r/PHGamers</t>
+          <t>r/StopGaming</t>
         </is>
       </c>
       <c r="C884" s="3" t="inlineStr">
@@ -55711,12 +55711,12 @@
       </c>
       <c r="F884" s="3" t="inlineStr">
         <is>
-          <t>Philippine player sentiment across console, PC, mobile, and VR. The largest national gaming subreddit outside Europe, consistent with the Philippines' English-language position.</t>
+          <t>Compulsive play and recovery in the first person. The addiction and screen-time discourse from the people it is about, rather than from clinicians or the press.</t>
         </is>
       </c>
       <c r="G884" s="3" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="H884" s="3" t="inlineStr">
@@ -55731,7 +55731,7 @@
       </c>
       <c r="J884" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/PHGamers</t>
+          <t>https://www.reddit.com/r/StopGaming/</t>
         </is>
       </c>
       <c r="K884" s="3" t="inlineStr"/>
@@ -55746,12 +55746,12 @@
     <row r="885">
       <c r="A885" s="3" t="inlineStr">
         <is>
-          <t>r-indogamer</t>
+          <t>r-emulation</t>
         </is>
       </c>
       <c r="B885" s="3" t="inlineStr">
         <is>
-          <t>r/IndoGamer</t>
+          <t>r/emulation</t>
         </is>
       </c>
       <c r="C885" s="3" t="inlineStr">
@@ -55771,12 +55771,12 @@
       </c>
       <c r="F885" s="3" t="inlineStr">
         <is>
-          <t>Indonesian player sentiment, predominantly in English. The local-language conversation sits on Kaskus, so this is the English-language layer only.</t>
+          <t>Emulation news and the preservation and legality arguments around it. Where the digital preservation fight is followed by the people doing the preserving.</t>
         </is>
       </c>
       <c r="G885" s="3" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="H885" s="3" t="inlineStr">
@@ -55791,7 +55791,7 @@
       </c>
       <c r="J885" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/IndoGamer</t>
+          <t>https://www.reddit.com/r/emulation/</t>
         </is>
       </c>
       <c r="K885" s="3" t="inlineStr"/>
@@ -55806,12 +55806,12 @@
     <row r="886">
       <c r="A886" s="3" t="inlineStr">
         <is>
-          <t>r-vietnamgaming</t>
+          <t>r-virtualreality</t>
         </is>
       </c>
       <c r="B886" s="3" t="inlineStr">
         <is>
-          <t>r/VietnamGaming</t>
+          <t>r/virtualreality</t>
         </is>
       </c>
       <c r="C886" s="3" t="inlineStr">
@@ -55831,12 +55831,12 @@
       </c>
       <c r="F886" s="3" t="inlineStr">
         <is>
-          <t>Vietnamese scene discussion, procurement, and gameplay, primarily in English. The local-language conversation sits on VOZ, so this is the English-language layer only.</t>
+          <t>Headset-agnostic VR discussion, buying advice and troubleshooting. A read on whether VR is growing, from owners rather than vendors.</t>
         </is>
       </c>
       <c r="G886" s="3" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="H886" s="3" t="inlineStr">
@@ -55851,7 +55851,7 @@
       </c>
       <c r="J886" s="3" t="inlineStr">
         <is>
-          <t>https://www.reddit.com/r/VietnamGaming</t>
+          <t>https://www.reddit.com/r/virtualreality/</t>
         </is>
       </c>
       <c r="K886" s="3" t="inlineStr"/>
@@ -55866,12 +55866,12 @@
     <row r="887">
       <c r="A887" s="3" t="inlineStr">
         <is>
-          <t>game8</t>
+          <t>r-twitch</t>
         </is>
       </c>
       <c r="B887" s="3" t="inlineStr">
         <is>
-          <t>Game8 (ゲームエイト)</t>
+          <t>r/Twitch</t>
         </is>
       </c>
       <c r="C887" s="3" t="inlineStr">
@@ -55886,22 +55886,22 @@
       </c>
       <c r="E887" s="3" t="inlineStr">
         <is>
-          <t>Walkthrough and guide site</t>
+          <t>Subreddit</t>
         </is>
       </c>
       <c r="F887" s="3" t="inlineStr">
         <is>
-          <t>Japan's largest walkthrough media by its own count (42 million monthly unique users, up to 500 million page views), a 100% Gunosy subsidiary with an English edition. Traffic per title is a proxy for which mobile and console games have active players. Guide sites are ad-funded and built to rank in search, so read traffic as engagement, not sentiment.</t>
+          <t>Streamers on the platform's rules, payouts and tooling. The creator economy from the small-creator side, where a platform change lands as income.</t>
         </is>
       </c>
       <c r="G887" s="3" t="inlineStr">
         <is>
-          <t>JP</t>
+          <t>US</t>
         </is>
       </c>
       <c r="H887" s="3" t="inlineStr">
         <is>
-          <t>Japanese</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I887" s="3" t="inlineStr">
@@ -55911,7 +55911,7 @@
       </c>
       <c r="J887" s="3" t="inlineStr">
         <is>
-          <t>https://game8.jp/</t>
+          <t>https://www.reddit.com/r/Twitch/</t>
         </is>
       </c>
       <c r="K887" s="3" t="inlineStr"/>
@@ -55926,12 +55926,12 @@
     <row r="888">
       <c r="A888" s="3" t="inlineStr">
         <is>
-          <t>gamewith</t>
+          <t>r-cozygamers</t>
         </is>
       </c>
       <c r="B888" s="3" t="inlineStr">
         <is>
-          <t>GameWith (ゲームウィズ)</t>
+          <t>r/CozyGamers</t>
         </is>
       </c>
       <c r="C888" s="3" t="inlineStr">
@@ -55946,22 +55946,22 @@
       </c>
       <c r="E888" s="3" t="inlineStr">
         <is>
-          <t>Walkthrough and guide site</t>
+          <t>Subreddit</t>
         </is>
       </c>
       <c r="F888" s="3" t="inlineStr">
         <is>
-          <t>The other national-scale guide site, run by GameWith, Inc., listed on the Tokyo Stock Exchange (6552) since 2017 and so the one guide business with public accounts; its results are a window on the guide-media economy, and it has expanded into esports and a gamer ISP.</t>
+          <t>Cozy and relaxing games, one of the fastest-growing gaming subs, with an adult and largely female audience. The cozy genre's own venue.</t>
         </is>
       </c>
       <c r="G888" s="3" t="inlineStr">
         <is>
-          <t>JP</t>
+          <t>US</t>
         </is>
       </c>
       <c r="H888" s="3" t="inlineStr">
         <is>
-          <t>Japanese</t>
+          <t>English</t>
         </is>
       </c>
       <c r="I888" s="3" t="inlineStr">
@@ -55971,7 +55971,7 @@
       </c>
       <c r="J888" s="3" t="inlineStr">
         <is>
-          <t>https://gamewith.jp/</t>
+          <t>https://www.reddit.com/r/CozyGamers/</t>
         </is>
       </c>
       <c r="K888" s="3" t="inlineStr"/>
@@ -55983,8 +55983,1628 @@
       <c r="Q888" s="3" t="inlineStr"/>
       <c r="R888" s="3" t="inlineStr"/>
     </row>
+    <row r="889">
+      <c r="A889" s="3" t="inlineStr">
+        <is>
+          <t>r-zocken</t>
+        </is>
+      </c>
+      <c r="B889" s="3" t="inlineStr">
+        <is>
+          <t>r/zocken</t>
+        </is>
+      </c>
+      <c r="C889" s="3" t="inlineStr">
+        <is>
+          <t>Communities</t>
+        </is>
+      </c>
+      <c r="D889" s="3" t="inlineStr">
+        <is>
+          <t>Forum or community</t>
+        </is>
+      </c>
+      <c r="E889" s="3" t="inlineStr">
+        <is>
+          <t>Subreddit</t>
+        </is>
+      </c>
+      <c r="F889" s="3" t="inlineStr">
+        <is>
+          <t>General German-language player sentiment and discussion. The venue for German community temperature on Reddit, not r/de. Never for citation. The main German-language gaming community.</t>
+        </is>
+      </c>
+      <c r="G889" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="H889" s="3" t="inlineStr">
+        <is>
+          <t>German</t>
+        </is>
+      </c>
+      <c r="I889" s="3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="J889" s="3" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/zocken</t>
+        </is>
+      </c>
+      <c r="K889" s="3" t="inlineStr"/>
+      <c r="L889" s="3" t="inlineStr"/>
+      <c r="M889" s="3" t="inlineStr"/>
+      <c r="N889" s="3" t="inlineStr"/>
+      <c r="O889" s="3" t="inlineStr"/>
+      <c r="P889" s="3" t="inlineStr"/>
+      <c r="Q889" s="3" t="inlineStr"/>
+      <c r="R889" s="3" t="inlineStr"/>
+    </row>
+    <row r="890">
+      <c r="A890" s="3" t="inlineStr">
+        <is>
+          <t>r-pcgamingde</t>
+        </is>
+      </c>
+      <c r="B890" s="3" t="inlineStr">
+        <is>
+          <t>r/PCGamingDE</t>
+        </is>
+      </c>
+      <c r="C890" s="3" t="inlineStr">
+        <is>
+          <t>Communities</t>
+        </is>
+      </c>
+      <c r="D890" s="3" t="inlineStr">
+        <is>
+          <t>Forum or community</t>
+        </is>
+      </c>
+      <c r="E890" s="3" t="inlineStr">
+        <is>
+          <t>Subreddit</t>
+        </is>
+      </c>
+      <c r="F890" s="3" t="inlineStr">
+        <is>
+          <t>German-language PC gaming discussion, builds, and platform sentiment.</t>
+        </is>
+      </c>
+      <c r="G890" s="3" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="H890" s="3" t="inlineStr">
+        <is>
+          <t>German</t>
+        </is>
+      </c>
+      <c r="I890" s="3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="J890" s="3" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/PCGamingDE</t>
+        </is>
+      </c>
+      <c r="K890" s="3" t="inlineStr"/>
+      <c r="L890" s="3" t="inlineStr"/>
+      <c r="M890" s="3" t="inlineStr"/>
+      <c r="N890" s="3" t="inlineStr"/>
+      <c r="O890" s="3" t="inlineStr"/>
+      <c r="P890" s="3" t="inlineStr"/>
+      <c r="Q890" s="3" t="inlineStr"/>
+      <c r="R890" s="3" t="inlineStr"/>
+    </row>
+    <row r="891">
+      <c r="A891" s="3" t="inlineStr">
+        <is>
+          <t>r-jeuxvideo</t>
+        </is>
+      </c>
+      <c r="B891" s="3" t="inlineStr">
+        <is>
+          <t>r/jeuxvideo</t>
+        </is>
+      </c>
+      <c r="C891" s="3" t="inlineStr">
+        <is>
+          <t>Communities</t>
+        </is>
+      </c>
+      <c r="D891" s="3" t="inlineStr">
+        <is>
+          <t>Forum or community</t>
+        </is>
+      </c>
+      <c r="E891" s="3" t="inlineStr">
+        <is>
+          <t>Subreddit</t>
+        </is>
+      </c>
+      <c r="F891" s="3" t="inlineStr">
+        <is>
+          <t>The main French-language gaming community. French player sentiment and discussion at scale, including esports threads. Not affiliated with the Webedia site jeuxvideo.com despite the shared name.</t>
+        </is>
+      </c>
+      <c r="G891" s="3" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="H891" s="3" t="inlineStr">
+        <is>
+          <t>French</t>
+        </is>
+      </c>
+      <c r="I891" s="3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="J891" s="3" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/jeuxvideo</t>
+        </is>
+      </c>
+      <c r="K891" s="3" t="inlineStr"/>
+      <c r="L891" s="3" t="inlineStr"/>
+      <c r="M891" s="3" t="inlineStr"/>
+      <c r="N891" s="3" t="inlineStr"/>
+      <c r="O891" s="3" t="inlineStr"/>
+      <c r="P891" s="3" t="inlineStr"/>
+      <c r="Q891" s="3" t="inlineStr"/>
+      <c r="R891" s="3" t="inlineStr"/>
+    </row>
+    <row r="892">
+      <c r="A892" s="3" t="inlineStr">
+        <is>
+          <t>r-italygames</t>
+        </is>
+      </c>
+      <c r="B892" s="3" t="inlineStr">
+        <is>
+          <t>r/italygames</t>
+        </is>
+      </c>
+      <c r="C892" s="3" t="inlineStr">
+        <is>
+          <t>Communities</t>
+        </is>
+      </c>
+      <c r="D892" s="3" t="inlineStr">
+        <is>
+          <t>Forum or community</t>
+        </is>
+      </c>
+      <c r="E892" s="3" t="inlineStr">
+        <is>
+          <t>Subreddit</t>
+        </is>
+      </c>
+      <c r="F892" s="3" t="inlineStr">
+        <is>
+          <t>Italian player sentiment across PC, console, retro, and tabletop. The venue for Italian community temperature on Reddit, not r/italy. The main Italian gaming community.</t>
+        </is>
+      </c>
+      <c r="G892" s="3" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="H892" s="3" t="inlineStr">
+        <is>
+          <t>Italian</t>
+        </is>
+      </c>
+      <c r="I892" s="3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="J892" s="3" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/italygames</t>
+        </is>
+      </c>
+      <c r="K892" s="3" t="inlineStr"/>
+      <c r="L892" s="3" t="inlineStr"/>
+      <c r="M892" s="3" t="inlineStr"/>
+      <c r="N892" s="3" t="inlineStr"/>
+      <c r="O892" s="3" t="inlineStr"/>
+      <c r="P892" s="3" t="inlineStr"/>
+      <c r="Q892" s="3" t="inlineStr"/>
+      <c r="R892" s="3" t="inlineStr"/>
+    </row>
+    <row r="893">
+      <c r="A893" s="3" t="inlineStr">
+        <is>
+          <t>r-gamedevelopersitaly</t>
+        </is>
+      </c>
+      <c r="B893" s="3" t="inlineStr">
+        <is>
+          <t>r/GameDevelopersItaly</t>
+        </is>
+      </c>
+      <c r="C893" s="3" t="inlineStr">
+        <is>
+          <t>Communities</t>
+        </is>
+      </c>
+      <c r="D893" s="3" t="inlineStr">
+        <is>
+          <t>Forum or community</t>
+        </is>
+      </c>
+      <c r="E893" s="3" t="inlineStr">
+        <is>
+          <t>Subreddit</t>
+        </is>
+      </c>
+      <c r="F893" s="3" t="inlineStr">
+        <is>
+          <t>Italian-language developer discussion. Useful as a window on the Italian dev scene, which has no trade press.</t>
+        </is>
+      </c>
+      <c r="G893" s="3" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="H893" s="3" t="inlineStr">
+        <is>
+          <t>Italian</t>
+        </is>
+      </c>
+      <c r="I893" s="3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="J893" s="3" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/GameDevelopersItaly</t>
+        </is>
+      </c>
+      <c r="K893" s="3" t="inlineStr"/>
+      <c r="L893" s="3" t="inlineStr"/>
+      <c r="M893" s="3" t="inlineStr"/>
+      <c r="N893" s="3" t="inlineStr"/>
+      <c r="O893" s="3" t="inlineStr"/>
+      <c r="P893" s="3" t="inlineStr"/>
+      <c r="Q893" s="3" t="inlineStr"/>
+      <c r="R893" s="3" t="inlineStr"/>
+    </row>
+    <row r="894">
+      <c r="A894" s="3" t="inlineStr">
+        <is>
+          <t>r-gamesecultura</t>
+        </is>
+      </c>
+      <c r="B894" s="3" t="inlineStr">
+        <is>
+          <t>r/gamesEcultura</t>
+        </is>
+      </c>
+      <c r="C894" s="3" t="inlineStr">
+        <is>
+          <t>Communities</t>
+        </is>
+      </c>
+      <c r="D894" s="3" t="inlineStr">
+        <is>
+          <t>Forum or community</t>
+        </is>
+      </c>
+      <c r="E894" s="3" t="inlineStr">
+        <is>
+          <t>Subreddit</t>
+        </is>
+      </c>
+      <c r="F894" s="3" t="inlineStr">
+        <is>
+          <t>Brazilian player sentiment where games meet wider geek culture. The biggest Reddit venue for Brazilian community temperature. The largest Brazilian gaming community.</t>
+        </is>
+      </c>
+      <c r="G894" s="3" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="H894" s="3" t="inlineStr">
+        <is>
+          <t>Portuguese</t>
+        </is>
+      </c>
+      <c r="I894" s="3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="J894" s="3" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/gamesEcultura</t>
+        </is>
+      </c>
+      <c r="K894" s="3" t="inlineStr"/>
+      <c r="L894" s="3" t="inlineStr"/>
+      <c r="M894" s="3" t="inlineStr"/>
+      <c r="N894" s="3" t="inlineStr"/>
+      <c r="O894" s="3" t="inlineStr"/>
+      <c r="P894" s="3" t="inlineStr"/>
+      <c r="Q894" s="3" t="inlineStr"/>
+      <c r="R894" s="3" t="inlineStr"/>
+    </row>
+    <row r="895">
+      <c r="A895" s="3" t="inlineStr">
+        <is>
+          <t>r-jogosbrasil</t>
+        </is>
+      </c>
+      <c r="B895" s="3" t="inlineStr">
+        <is>
+          <t>r/jogosbrasil</t>
+        </is>
+      </c>
+      <c r="C895" s="3" t="inlineStr">
+        <is>
+          <t>Communities</t>
+        </is>
+      </c>
+      <c r="D895" s="3" t="inlineStr">
+        <is>
+          <t>Forum or community</t>
+        </is>
+      </c>
+      <c r="E895" s="3" t="inlineStr">
+        <is>
+          <t>Subreddit</t>
+        </is>
+      </c>
+      <c r="F895" s="3" t="inlineStr">
+        <is>
+          <t>Brazilian discussion of PC, console, and mobile games plus release and free-game news.</t>
+        </is>
+      </c>
+      <c r="G895" s="3" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="H895" s="3" t="inlineStr">
+        <is>
+          <t>Portuguese</t>
+        </is>
+      </c>
+      <c r="I895" s="3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="J895" s="3" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/jogosbrasil</t>
+        </is>
+      </c>
+      <c r="K895" s="3" t="inlineStr"/>
+      <c r="L895" s="3" t="inlineStr"/>
+      <c r="M895" s="3" t="inlineStr"/>
+      <c r="N895" s="3" t="inlineStr"/>
+      <c r="O895" s="3" t="inlineStr"/>
+      <c r="P895" s="3" t="inlineStr"/>
+      <c r="Q895" s="3" t="inlineStr"/>
+      <c r="R895" s="3" t="inlineStr"/>
+    </row>
+    <row r="896">
+      <c r="A896" s="3" t="inlineStr">
+        <is>
+          <t>r-playstationbrasil</t>
+        </is>
+      </c>
+      <c r="B896" s="3" t="inlineStr">
+        <is>
+          <t>r/playstationbrasil</t>
+        </is>
+      </c>
+      <c r="C896" s="3" t="inlineStr">
+        <is>
+          <t>Communities</t>
+        </is>
+      </c>
+      <c r="D896" s="3" t="inlineStr">
+        <is>
+          <t>Forum or community</t>
+        </is>
+      </c>
+      <c r="E896" s="3" t="inlineStr">
+        <is>
+          <t>Subreddit</t>
+        </is>
+      </c>
+      <c r="F896" s="3" t="inlineStr">
+        <is>
+          <t>Brazilian platform-specific sentiment, pricing complaints, and buying culture on PlayStation.</t>
+        </is>
+      </c>
+      <c r="G896" s="3" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="H896" s="3" t="inlineStr">
+        <is>
+          <t>Portuguese</t>
+        </is>
+      </c>
+      <c r="I896" s="3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="J896" s="3" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/playstationbrasil</t>
+        </is>
+      </c>
+      <c r="K896" s="3" t="inlineStr"/>
+      <c r="L896" s="3" t="inlineStr"/>
+      <c r="M896" s="3" t="inlineStr"/>
+      <c r="N896" s="3" t="inlineStr"/>
+      <c r="O896" s="3" t="inlineStr"/>
+      <c r="P896" s="3" t="inlineStr"/>
+      <c r="Q896" s="3" t="inlineStr"/>
+      <c r="R896" s="3" t="inlineStr"/>
+    </row>
+    <row r="897">
+      <c r="A897" s="3" t="inlineStr">
+        <is>
+          <t>r-jogatina</t>
+        </is>
+      </c>
+      <c r="B897" s="3" t="inlineStr">
+        <is>
+          <t>r/jogatina</t>
+        </is>
+      </c>
+      <c r="C897" s="3" t="inlineStr">
+        <is>
+          <t>Communities</t>
+        </is>
+      </c>
+      <c r="D897" s="3" t="inlineStr">
+        <is>
+          <t>Forum or community</t>
+        </is>
+      </c>
+      <c r="E897" s="3" t="inlineStr">
+        <is>
+          <t>Subreddit</t>
+        </is>
+      </c>
+      <c r="F897" s="3" t="inlineStr">
+        <is>
+          <t>Brazilian general games discussion.</t>
+        </is>
+      </c>
+      <c r="G897" s="3" t="inlineStr">
+        <is>
+          <t>BR</t>
+        </is>
+      </c>
+      <c r="H897" s="3" t="inlineStr">
+        <is>
+          <t>Portuguese</t>
+        </is>
+      </c>
+      <c r="I897" s="3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="J897" s="3" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/jogatina</t>
+        </is>
+      </c>
+      <c r="K897" s="3" t="inlineStr"/>
+      <c r="L897" s="3" t="inlineStr"/>
+      <c r="M897" s="3" t="inlineStr"/>
+      <c r="N897" s="3" t="inlineStr"/>
+      <c r="O897" s="3" t="inlineStr"/>
+      <c r="P897" s="3" t="inlineStr"/>
+      <c r="Q897" s="3" t="inlineStr"/>
+      <c r="R897" s="3" t="inlineStr"/>
+    </row>
+    <row r="898">
+      <c r="A898" s="3" t="inlineStr">
+        <is>
+          <t>r-videojuegosmx</t>
+        </is>
+      </c>
+      <c r="B898" s="3" t="inlineStr">
+        <is>
+          <t>r/VideojuegosMX</t>
+        </is>
+      </c>
+      <c r="C898" s="3" t="inlineStr">
+        <is>
+          <t>Communities</t>
+        </is>
+      </c>
+      <c r="D898" s="3" t="inlineStr">
+        <is>
+          <t>Forum or community</t>
+        </is>
+      </c>
+      <c r="E898" s="3" t="inlineStr">
+        <is>
+          <t>Subreddit</t>
+        </is>
+      </c>
+      <c r="F898" s="3" t="inlineStr">
+        <is>
+          <t>Mexican player sentiment and discussion.</t>
+        </is>
+      </c>
+      <c r="G898" s="3" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="H898" s="3" t="inlineStr">
+        <is>
+          <t>Spanish</t>
+        </is>
+      </c>
+      <c r="I898" s="3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="J898" s="3" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/VideojuegosMX</t>
+        </is>
+      </c>
+      <c r="K898" s="3" t="inlineStr"/>
+      <c r="L898" s="3" t="inlineStr"/>
+      <c r="M898" s="3" t="inlineStr"/>
+      <c r="N898" s="3" t="inlineStr"/>
+      <c r="O898" s="3" t="inlineStr"/>
+      <c r="P898" s="3" t="inlineStr"/>
+      <c r="Q898" s="3" t="inlineStr"/>
+      <c r="R898" s="3" t="inlineStr"/>
+    </row>
+    <row r="899">
+      <c r="A899" s="3" t="inlineStr">
+        <is>
+          <t>r-videojuegos</t>
+        </is>
+      </c>
+      <c r="B899" s="3" t="inlineStr">
+        <is>
+          <t>r/videojuegos</t>
+        </is>
+      </c>
+      <c r="C899" s="3" t="inlineStr">
+        <is>
+          <t>Communities</t>
+        </is>
+      </c>
+      <c r="D899" s="3" t="inlineStr">
+        <is>
+          <t>Forum or community</t>
+        </is>
+      </c>
+      <c r="E899" s="3" t="inlineStr">
+        <is>
+          <t>Subreddit</t>
+        </is>
+      </c>
+      <c r="F899" s="3" t="inlineStr">
+        <is>
+          <t>Spanish-language player sentiment across Spain and Latin America. A language venue rather than a country venue, so read alongside the national subs.</t>
+        </is>
+      </c>
+      <c r="G899" s="3" t="inlineStr">
+        <is>
+          <t>ES; LATAM; MX</t>
+        </is>
+      </c>
+      <c r="H899" s="3" t="inlineStr">
+        <is>
+          <t>Spanish</t>
+        </is>
+      </c>
+      <c r="I899" s="3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="J899" s="3" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/videojuegos/</t>
+        </is>
+      </c>
+      <c r="K899" s="3" t="inlineStr"/>
+      <c r="L899" s="3" t="inlineStr"/>
+      <c r="M899" s="3" t="inlineStr"/>
+      <c r="N899" s="3" t="inlineStr"/>
+      <c r="O899" s="3" t="inlineStr"/>
+      <c r="P899" s="3" t="inlineStr"/>
+      <c r="Q899" s="3" t="inlineStr"/>
+      <c r="R899" s="3" t="inlineStr"/>
+    </row>
+    <row r="900">
+      <c r="A900" s="3" t="inlineStr">
+        <is>
+          <t>r-esgaming</t>
+        </is>
+      </c>
+      <c r="B900" s="3" t="inlineStr">
+        <is>
+          <t>r/esGaming</t>
+        </is>
+      </c>
+      <c r="C900" s="3" t="inlineStr">
+        <is>
+          <t>Communities</t>
+        </is>
+      </c>
+      <c r="D900" s="3" t="inlineStr">
+        <is>
+          <t>Forum or community</t>
+        </is>
+      </c>
+      <c r="E900" s="3" t="inlineStr">
+        <is>
+          <t>Subreddit</t>
+        </is>
+      </c>
+      <c r="F900" s="3" t="inlineStr">
+        <is>
+          <t>Spanish player sentiment and discussion at scale. Sits alongside the Mediavida forum rather than replacing it.</t>
+        </is>
+      </c>
+      <c r="G900" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="H900" s="3" t="inlineStr">
+        <is>
+          <t>Spanish</t>
+        </is>
+      </c>
+      <c r="I900" s="3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="J900" s="3" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/esGaming</t>
+        </is>
+      </c>
+      <c r="K900" s="3" t="inlineStr"/>
+      <c r="L900" s="3" t="inlineStr"/>
+      <c r="M900" s="3" t="inlineStr"/>
+      <c r="N900" s="3" t="inlineStr"/>
+      <c r="O900" s="3" t="inlineStr"/>
+      <c r="P900" s="3" t="inlineStr"/>
+      <c r="Q900" s="3" t="inlineStr"/>
+      <c r="R900" s="3" t="inlineStr"/>
+    </row>
+    <row r="901">
+      <c r="A901" s="3" t="inlineStr">
+        <is>
+          <t>r-geymingtr</t>
+        </is>
+      </c>
+      <c r="B901" s="3" t="inlineStr">
+        <is>
+          <t>r/GeymingTr</t>
+        </is>
+      </c>
+      <c r="C901" s="3" t="inlineStr">
+        <is>
+          <t>Communities</t>
+        </is>
+      </c>
+      <c r="D901" s="3" t="inlineStr">
+        <is>
+          <t>Forum or community</t>
+        </is>
+      </c>
+      <c r="E901" s="3" t="inlineStr">
+        <is>
+          <t>Subreddit</t>
+        </is>
+      </c>
+      <c r="F901" s="3" t="inlineStr">
+        <is>
+          <t>Turkish player sentiment in a casual register. The name is a phonetic spelling of gaming, an instance of the English loanword doing the work the betting-polluted word oyun cannot.</t>
+        </is>
+      </c>
+      <c r="G901" s="3" t="inlineStr">
+        <is>
+          <t>TR</t>
+        </is>
+      </c>
+      <c r="H901" s="3" t="inlineStr">
+        <is>
+          <t>Turkish</t>
+        </is>
+      </c>
+      <c r="I901" s="3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="J901" s="3" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/GeymingTr</t>
+        </is>
+      </c>
+      <c r="K901" s="3" t="inlineStr"/>
+      <c r="L901" s="3" t="inlineStr"/>
+      <c r="M901" s="3" t="inlineStr"/>
+      <c r="N901" s="3" t="inlineStr"/>
+      <c r="O901" s="3" t="inlineStr"/>
+      <c r="P901" s="3" t="inlineStr"/>
+      <c r="Q901" s="3" t="inlineStr"/>
+      <c r="R901" s="3" t="inlineStr"/>
+    </row>
+    <row r="902">
+      <c r="A902" s="3" t="inlineStr">
+        <is>
+          <t>r-oyun</t>
+        </is>
+      </c>
+      <c r="B902" s="3" t="inlineStr">
+        <is>
+          <t>r/oyun</t>
+        </is>
+      </c>
+      <c r="C902" s="3" t="inlineStr">
+        <is>
+          <t>Communities</t>
+        </is>
+      </c>
+      <c r="D902" s="3" t="inlineStr">
+        <is>
+          <t>Forum or community</t>
+        </is>
+      </c>
+      <c r="E902" s="3" t="inlineStr">
+        <is>
+          <t>Subreddit</t>
+        </is>
+      </c>
+      <c r="F902" s="3" t="inlineStr">
+        <is>
+          <t>Turkish general games discussion, the second general venue alongside r/GeymingTr.</t>
+        </is>
+      </c>
+      <c r="G902" s="3" t="inlineStr">
+        <is>
+          <t>TR</t>
+        </is>
+      </c>
+      <c r="H902" s="3" t="inlineStr">
+        <is>
+          <t>Turkish</t>
+        </is>
+      </c>
+      <c r="I902" s="3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="J902" s="3" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/oyun</t>
+        </is>
+      </c>
+      <c r="K902" s="3" t="inlineStr"/>
+      <c r="L902" s="3" t="inlineStr"/>
+      <c r="M902" s="3" t="inlineStr"/>
+      <c r="N902" s="3" t="inlineStr"/>
+      <c r="O902" s="3" t="inlineStr"/>
+      <c r="P902" s="3" t="inlineStr"/>
+      <c r="Q902" s="3" t="inlineStr"/>
+      <c r="R902" s="3" t="inlineStr"/>
+    </row>
+    <row r="903">
+      <c r="A903" s="3" t="inlineStr">
+        <is>
+          <t>r-trgamedeveloper</t>
+        </is>
+      </c>
+      <c r="B903" s="3" t="inlineStr">
+        <is>
+          <t>r/TrGameDeveloper</t>
+        </is>
+      </c>
+      <c r="C903" s="3" t="inlineStr">
+        <is>
+          <t>Communities</t>
+        </is>
+      </c>
+      <c r="D903" s="3" t="inlineStr">
+        <is>
+          <t>Forum or community</t>
+        </is>
+      </c>
+      <c r="E903" s="3" t="inlineStr">
+        <is>
+          <t>Subreddit</t>
+        </is>
+      </c>
+      <c r="F903" s="3" t="inlineStr">
+        <is>
+          <t>Turkish developer discussion and publishing help. The largest gamedev subreddit found, consistent with Turkey's production-market profile.</t>
+        </is>
+      </c>
+      <c r="G903" s="3" t="inlineStr">
+        <is>
+          <t>TR</t>
+        </is>
+      </c>
+      <c r="H903" s="3" t="inlineStr">
+        <is>
+          <t>Turkish</t>
+        </is>
+      </c>
+      <c r="I903" s="3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="J903" s="3" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/TrGameDeveloper</t>
+        </is>
+      </c>
+      <c r="K903" s="3" t="inlineStr"/>
+      <c r="L903" s="3" t="inlineStr"/>
+      <c r="M903" s="3" t="inlineStr"/>
+      <c r="N903" s="3" t="inlineStr"/>
+      <c r="O903" s="3" t="inlineStr"/>
+      <c r="P903" s="3" t="inlineStr"/>
+      <c r="Q903" s="3" t="inlineStr"/>
+      <c r="R903" s="3" t="inlineStr"/>
+    </row>
+    <row r="904">
+      <c r="A904" s="3" t="inlineStr">
+        <is>
+          <t>r-turkoyunsektoru</t>
+        </is>
+      </c>
+      <c r="B904" s="3" t="inlineStr">
+        <is>
+          <t>r/TurkOyunSektoru</t>
+        </is>
+      </c>
+      <c r="C904" s="3" t="inlineStr">
+        <is>
+          <t>Communities</t>
+        </is>
+      </c>
+      <c r="D904" s="3" t="inlineStr">
+        <is>
+          <t>Forum or community</t>
+        </is>
+      </c>
+      <c r="E904" s="3" t="inlineStr">
+        <is>
+          <t>Subreddit</t>
+        </is>
+      </c>
+      <c r="F904" s="3" t="inlineStr">
+        <is>
+          <t>Turkish industry and publishing discussion, the business side of the scene r/TrGameDeveloper covers from the craft side.</t>
+        </is>
+      </c>
+      <c r="G904" s="3" t="inlineStr">
+        <is>
+          <t>TR</t>
+        </is>
+      </c>
+      <c r="H904" s="3" t="inlineStr">
+        <is>
+          <t>Turkish</t>
+        </is>
+      </c>
+      <c r="I904" s="3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="J904" s="3" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/TurkOyunSektoru</t>
+        </is>
+      </c>
+      <c r="K904" s="3" t="inlineStr"/>
+      <c r="L904" s="3" t="inlineStr"/>
+      <c r="M904" s="3" t="inlineStr"/>
+      <c r="N904" s="3" t="inlineStr"/>
+      <c r="O904" s="3" t="inlineStr"/>
+      <c r="P904" s="3" t="inlineStr"/>
+      <c r="Q904" s="3" t="inlineStr"/>
+      <c r="R904" s="3" t="inlineStr"/>
+    </row>
+    <row r="905">
+      <c r="A905" s="3" t="inlineStr">
+        <is>
+          <t>r-saudi-gamers</t>
+        </is>
+      </c>
+      <c r="B905" s="3" t="inlineStr">
+        <is>
+          <t>r/saudi_gamers</t>
+        </is>
+      </c>
+      <c r="C905" s="3" t="inlineStr">
+        <is>
+          <t>Communities</t>
+        </is>
+      </c>
+      <c r="D905" s="3" t="inlineStr">
+        <is>
+          <t>Forum or community</t>
+        </is>
+      </c>
+      <c r="E905" s="3" t="inlineStr">
+        <is>
+          <t>Subreddit</t>
+        </is>
+      </c>
+      <c r="F905" s="3" t="inlineStr">
+        <is>
+          <t>Saudi and pan-Arab player sentiment. One of the few venues in the MENA stack with no institutional or state-linked owner.</t>
+        </is>
+      </c>
+      <c r="G905" s="3" t="inlineStr">
+        <is>
+          <t>MENA</t>
+        </is>
+      </c>
+      <c r="H905" s="3" t="inlineStr">
+        <is>
+          <t>Arabic</t>
+        </is>
+      </c>
+      <c r="I905" s="3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="J905" s="3" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/saudi_gamers</t>
+        </is>
+      </c>
+      <c r="K905" s="3" t="inlineStr"/>
+      <c r="L905" s="3" t="inlineStr"/>
+      <c r="M905" s="3" t="inlineStr"/>
+      <c r="N905" s="3" t="inlineStr"/>
+      <c r="O905" s="3" t="inlineStr"/>
+      <c r="P905" s="3" t="inlineStr"/>
+      <c r="Q905" s="3" t="inlineStr"/>
+      <c r="R905" s="3" t="inlineStr"/>
+    </row>
+    <row r="906">
+      <c r="A906" s="3" t="inlineStr">
+        <is>
+          <t>r-iraqigamers</t>
+        </is>
+      </c>
+      <c r="B906" s="3" t="inlineStr">
+        <is>
+          <t>r/Iraqigamers</t>
+        </is>
+      </c>
+      <c r="C906" s="3" t="inlineStr">
+        <is>
+          <t>Communities</t>
+        </is>
+      </c>
+      <c r="D906" s="3" t="inlineStr">
+        <is>
+          <t>Forum or community</t>
+        </is>
+      </c>
+      <c r="E906" s="3" t="inlineStr">
+        <is>
+          <t>Subreddit</t>
+        </is>
+      </c>
+      <c r="F906" s="3" t="inlineStr">
+        <is>
+          <t>Iraqi player sentiment and memes.</t>
+        </is>
+      </c>
+      <c r="G906" s="3" t="inlineStr">
+        <is>
+          <t>MENA</t>
+        </is>
+      </c>
+      <c r="H906" s="3" t="inlineStr">
+        <is>
+          <t>Arabic</t>
+        </is>
+      </c>
+      <c r="I906" s="3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="J906" s="3" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/Iraqigamers</t>
+        </is>
+      </c>
+      <c r="K906" s="3" t="inlineStr"/>
+      <c r="L906" s="3" t="inlineStr"/>
+      <c r="M906" s="3" t="inlineStr"/>
+      <c r="N906" s="3" t="inlineStr"/>
+      <c r="O906" s="3" t="inlineStr"/>
+      <c r="P906" s="3" t="inlineStr"/>
+      <c r="Q906" s="3" t="inlineStr"/>
+      <c r="R906" s="3" t="inlineStr"/>
+    </row>
+    <row r="907">
+      <c r="A907" s="3" t="inlineStr">
+        <is>
+          <t>r-egyptgaming-and-r-egyptgamingg</t>
+        </is>
+      </c>
+      <c r="B907" s="3" t="inlineStr">
+        <is>
+          <t>r/EgyptGaming and r/EgyptGaminGG</t>
+        </is>
+      </c>
+      <c r="C907" s="3" t="inlineStr">
+        <is>
+          <t>Communities</t>
+        </is>
+      </c>
+      <c r="D907" s="3" t="inlineStr">
+        <is>
+          <t>Forum or community</t>
+        </is>
+      </c>
+      <c r="E907" s="3" t="inlineStr">
+        <is>
+          <t>Subreddit</t>
+        </is>
+      </c>
+      <c r="F907" s="3" t="inlineStr">
+        <is>
+          <t>Egyptian player sentiment across two communities of similar size. Neither is clearly primary from outside, so both are listed.</t>
+        </is>
+      </c>
+      <c r="G907" s="3" t="inlineStr">
+        <is>
+          <t>MENA</t>
+        </is>
+      </c>
+      <c r="H907" s="3" t="inlineStr">
+        <is>
+          <t>Arabic</t>
+        </is>
+      </c>
+      <c r="I907" s="3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="J907" s="3" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/EgyptGaming</t>
+        </is>
+      </c>
+      <c r="K907" s="3" t="inlineStr"/>
+      <c r="L907" s="3" t="inlineStr"/>
+      <c r="M907" s="3" t="inlineStr"/>
+      <c r="N907" s="3" t="inlineStr"/>
+      <c r="O907" s="3" t="inlineStr"/>
+      <c r="P907" s="3" t="inlineStr"/>
+      <c r="Q907" s="3" t="inlineStr"/>
+      <c r="R907" s="3" t="inlineStr"/>
+    </row>
+    <row r="908">
+      <c r="A908" s="3" t="inlineStr">
+        <is>
+          <t>r-arabic-games</t>
+        </is>
+      </c>
+      <c r="B908" s="3" t="inlineStr">
+        <is>
+          <t>r/Arabic_Games</t>
+        </is>
+      </c>
+      <c r="C908" s="3" t="inlineStr">
+        <is>
+          <t>Communities</t>
+        </is>
+      </c>
+      <c r="D908" s="3" t="inlineStr">
+        <is>
+          <t>Forum or community</t>
+        </is>
+      </c>
+      <c r="E908" s="3" t="inlineStr">
+        <is>
+          <t>Subreddit</t>
+        </is>
+      </c>
+      <c r="F908" s="3" t="inlineStr">
+        <is>
+          <t>Arabic localization discourse, official and fan translations. Small but the only localization venue in this directory.</t>
+        </is>
+      </c>
+      <c r="G908" s="3" t="inlineStr">
+        <is>
+          <t>MENA</t>
+        </is>
+      </c>
+      <c r="H908" s="3" t="inlineStr">
+        <is>
+          <t>Arabic</t>
+        </is>
+      </c>
+      <c r="I908" s="3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="J908" s="3" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/Arabic_Games</t>
+        </is>
+      </c>
+      <c r="K908" s="3" t="inlineStr"/>
+      <c r="L908" s="3" t="inlineStr"/>
+      <c r="M908" s="3" t="inlineStr"/>
+      <c r="N908" s="3" t="inlineStr"/>
+      <c r="O908" s="3" t="inlineStr"/>
+      <c r="P908" s="3" t="inlineStr"/>
+      <c r="Q908" s="3" t="inlineStr"/>
+      <c r="R908" s="3" t="inlineStr"/>
+    </row>
+    <row r="909">
+      <c r="A909" s="3" t="inlineStr">
+        <is>
+          <t>r-spel</t>
+        </is>
+      </c>
+      <c r="B909" s="3" t="inlineStr">
+        <is>
+          <t>r/Spel</t>
+        </is>
+      </c>
+      <c r="C909" s="3" t="inlineStr">
+        <is>
+          <t>Communities</t>
+        </is>
+      </c>
+      <c r="D909" s="3" t="inlineStr">
+        <is>
+          <t>Forum or community</t>
+        </is>
+      </c>
+      <c r="E909" s="3" t="inlineStr">
+        <is>
+          <t>Subreddit</t>
+        </is>
+      </c>
+      <c r="F909" s="3" t="inlineStr">
+        <is>
+          <t>Swedish player sentiment, the one national-language venue in a bloc that otherwise uses English subreddits. The name reclaims the word spel, which in Swedish search otherwise pulls betting companies first.</t>
+        </is>
+      </c>
+      <c r="G909" s="3" t="inlineStr">
+        <is>
+          <t>Nordics</t>
+        </is>
+      </c>
+      <c r="H909" s="3" t="inlineStr">
+        <is>
+          <t>Swedish</t>
+        </is>
+      </c>
+      <c r="I909" s="3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="J909" s="3" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/Spel</t>
+        </is>
+      </c>
+      <c r="K909" s="3" t="inlineStr"/>
+      <c r="L909" s="3" t="inlineStr"/>
+      <c r="M909" s="3" t="inlineStr"/>
+      <c r="N909" s="3" t="inlineStr"/>
+      <c r="O909" s="3" t="inlineStr"/>
+      <c r="P909" s="3" t="inlineStr"/>
+      <c r="Q909" s="3" t="inlineStr"/>
+      <c r="R909" s="3" t="inlineStr"/>
+    </row>
+    <row r="910">
+      <c r="A910" s="3" t="inlineStr">
+        <is>
+          <t>dutch-gaming-reddit</t>
+        </is>
+      </c>
+      <c r="B910" s="3" t="inlineStr">
+        <is>
+          <t>Dutch gaming Reddit (r/GamingNL)</t>
+        </is>
+      </c>
+      <c r="C910" s="3" t="inlineStr">
+        <is>
+          <t>Communities</t>
+        </is>
+      </c>
+      <c r="D910" s="3" t="inlineStr">
+        <is>
+          <t>Forum or community</t>
+        </is>
+      </c>
+      <c r="E910" s="3" t="inlineStr">
+        <is>
+          <t>Subreddit</t>
+        </is>
+      </c>
+      <c r="F910" s="3" t="inlineStr">
+        <is>
+          <t>Dutch gamers use the international English subreddits, and the national sub r/GamingNL stays around 1.5K members in a country of 18 million.</t>
+        </is>
+      </c>
+      <c r="G910" s="3" t="inlineStr">
+        <is>
+          <t>NL</t>
+        </is>
+      </c>
+      <c r="H910" s="3" t="inlineStr">
+        <is>
+          <t>Dutch; English</t>
+        </is>
+      </c>
+      <c r="I910" s="3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="J910" s="3" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/GamingNL</t>
+        </is>
+      </c>
+      <c r="K910" s="3" t="inlineStr"/>
+      <c r="L910" s="3" t="inlineStr"/>
+      <c r="M910" s="3" t="inlineStr"/>
+      <c r="N910" s="3" t="inlineStr"/>
+      <c r="O910" s="3" t="inlineStr"/>
+      <c r="P910" s="3" t="inlineStr"/>
+      <c r="Q910" s="3" t="inlineStr"/>
+      <c r="R910" s="3" t="inlineStr"/>
+    </row>
+    <row r="911">
+      <c r="A911" s="3" t="inlineStr">
+        <is>
+          <t>r-phgamers</t>
+        </is>
+      </c>
+      <c r="B911" s="3" t="inlineStr">
+        <is>
+          <t>r/PHGamers</t>
+        </is>
+      </c>
+      <c r="C911" s="3" t="inlineStr">
+        <is>
+          <t>Communities</t>
+        </is>
+      </c>
+      <c r="D911" s="3" t="inlineStr">
+        <is>
+          <t>Forum or community</t>
+        </is>
+      </c>
+      <c r="E911" s="3" t="inlineStr">
+        <is>
+          <t>Subreddit</t>
+        </is>
+      </c>
+      <c r="F911" s="3" t="inlineStr">
+        <is>
+          <t>Philippine player sentiment across console, PC, mobile, and VR. The largest national gaming subreddit outside Europe, consistent with the Philippines' English-language position.</t>
+        </is>
+      </c>
+      <c r="G911" s="3" t="inlineStr">
+        <is>
+          <t>SEA</t>
+        </is>
+      </c>
+      <c r="H911" s="3" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="I911" s="3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="J911" s="3" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/PHGamers</t>
+        </is>
+      </c>
+      <c r="K911" s="3" t="inlineStr"/>
+      <c r="L911" s="3" t="inlineStr"/>
+      <c r="M911" s="3" t="inlineStr"/>
+      <c r="N911" s="3" t="inlineStr"/>
+      <c r="O911" s="3" t="inlineStr"/>
+      <c r="P911" s="3" t="inlineStr"/>
+      <c r="Q911" s="3" t="inlineStr"/>
+      <c r="R911" s="3" t="inlineStr"/>
+    </row>
+    <row r="912">
+      <c r="A912" s="3" t="inlineStr">
+        <is>
+          <t>r-indogamer</t>
+        </is>
+      </c>
+      <c r="B912" s="3" t="inlineStr">
+        <is>
+          <t>r/IndoGamer</t>
+        </is>
+      </c>
+      <c r="C912" s="3" t="inlineStr">
+        <is>
+          <t>Communities</t>
+        </is>
+      </c>
+      <c r="D912" s="3" t="inlineStr">
+        <is>
+          <t>Forum or community</t>
+        </is>
+      </c>
+      <c r="E912" s="3" t="inlineStr">
+        <is>
+          <t>Subreddit</t>
+        </is>
+      </c>
+      <c r="F912" s="3" t="inlineStr">
+        <is>
+          <t>Indonesian player sentiment, predominantly in English. The local-language conversation sits on Kaskus, so this is the English-language layer only.</t>
+        </is>
+      </c>
+      <c r="G912" s="3" t="inlineStr">
+        <is>
+          <t>SEA</t>
+        </is>
+      </c>
+      <c r="H912" s="3" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="I912" s="3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="J912" s="3" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/IndoGamer</t>
+        </is>
+      </c>
+      <c r="K912" s="3" t="inlineStr"/>
+      <c r="L912" s="3" t="inlineStr"/>
+      <c r="M912" s="3" t="inlineStr"/>
+      <c r="N912" s="3" t="inlineStr"/>
+      <c r="O912" s="3" t="inlineStr"/>
+      <c r="P912" s="3" t="inlineStr"/>
+      <c r="Q912" s="3" t="inlineStr"/>
+      <c r="R912" s="3" t="inlineStr"/>
+    </row>
+    <row r="913">
+      <c r="A913" s="3" t="inlineStr">
+        <is>
+          <t>r-vietnamgaming</t>
+        </is>
+      </c>
+      <c r="B913" s="3" t="inlineStr">
+        <is>
+          <t>r/VietnamGaming</t>
+        </is>
+      </c>
+      <c r="C913" s="3" t="inlineStr">
+        <is>
+          <t>Communities</t>
+        </is>
+      </c>
+      <c r="D913" s="3" t="inlineStr">
+        <is>
+          <t>Forum or community</t>
+        </is>
+      </c>
+      <c r="E913" s="3" t="inlineStr">
+        <is>
+          <t>Subreddit</t>
+        </is>
+      </c>
+      <c r="F913" s="3" t="inlineStr">
+        <is>
+          <t>Vietnamese scene discussion, procurement, and gameplay, primarily in English. The local-language conversation sits on VOZ, so this is the English-language layer only.</t>
+        </is>
+      </c>
+      <c r="G913" s="3" t="inlineStr">
+        <is>
+          <t>SEA</t>
+        </is>
+      </c>
+      <c r="H913" s="3" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="I913" s="3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="J913" s="3" t="inlineStr">
+        <is>
+          <t>https://www.reddit.com/r/VietnamGaming</t>
+        </is>
+      </c>
+      <c r="K913" s="3" t="inlineStr"/>
+      <c r="L913" s="3" t="inlineStr"/>
+      <c r="M913" s="3" t="inlineStr"/>
+      <c r="N913" s="3" t="inlineStr"/>
+      <c r="O913" s="3" t="inlineStr"/>
+      <c r="P913" s="3" t="inlineStr"/>
+      <c r="Q913" s="3" t="inlineStr"/>
+      <c r="R913" s="3" t="inlineStr"/>
+    </row>
+    <row r="914">
+      <c r="A914" s="3" t="inlineStr">
+        <is>
+          <t>game8</t>
+        </is>
+      </c>
+      <c r="B914" s="3" t="inlineStr">
+        <is>
+          <t>Game8 (ゲームエイト)</t>
+        </is>
+      </c>
+      <c r="C914" s="3" t="inlineStr">
+        <is>
+          <t>Communities</t>
+        </is>
+      </c>
+      <c r="D914" s="3" t="inlineStr">
+        <is>
+          <t>Forum or community</t>
+        </is>
+      </c>
+      <c r="E914" s="3" t="inlineStr">
+        <is>
+          <t>Walkthrough and guide site</t>
+        </is>
+      </c>
+      <c r="F914" s="3" t="inlineStr">
+        <is>
+          <t>Japan's largest walkthrough media by its own count (42 million monthly unique users, up to 500 million page views), a 100% Gunosy subsidiary with an English edition. Traffic per title is a proxy for which mobile and console games have active players. Guide sites are ad-funded and built to rank in search, so read traffic as engagement, not sentiment.</t>
+        </is>
+      </c>
+      <c r="G914" s="3" t="inlineStr">
+        <is>
+          <t>JP</t>
+        </is>
+      </c>
+      <c r="H914" s="3" t="inlineStr">
+        <is>
+          <t>Japanese</t>
+        </is>
+      </c>
+      <c r="I914" s="3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="J914" s="3" t="inlineStr">
+        <is>
+          <t>https://game8.jp/</t>
+        </is>
+      </c>
+      <c r="K914" s="3" t="inlineStr"/>
+      <c r="L914" s="3" t="inlineStr"/>
+      <c r="M914" s="3" t="inlineStr"/>
+      <c r="N914" s="3" t="inlineStr"/>
+      <c r="O914" s="3" t="inlineStr"/>
+      <c r="P914" s="3" t="inlineStr"/>
+      <c r="Q914" s="3" t="inlineStr"/>
+      <c r="R914" s="3" t="inlineStr"/>
+    </row>
+    <row r="915">
+      <c r="A915" s="3" t="inlineStr">
+        <is>
+          <t>gamewith</t>
+        </is>
+      </c>
+      <c r="B915" s="3" t="inlineStr">
+        <is>
+          <t>GameWith (ゲームウィズ)</t>
+        </is>
+      </c>
+      <c r="C915" s="3" t="inlineStr">
+        <is>
+          <t>Communities</t>
+        </is>
+      </c>
+      <c r="D915" s="3" t="inlineStr">
+        <is>
+          <t>Forum or community</t>
+        </is>
+      </c>
+      <c r="E915" s="3" t="inlineStr">
+        <is>
+          <t>Walkthrough and guide site</t>
+        </is>
+      </c>
+      <c r="F915" s="3" t="inlineStr">
+        <is>
+          <t>The other national-scale guide site, run by GameWith, Inc., listed on the Tokyo Stock Exchange (6552) since 2017 and so the one guide business with public accounts; its results are a window on the guide-media economy, and it has expanded into esports and a gamer ISP.</t>
+        </is>
+      </c>
+      <c r="G915" s="3" t="inlineStr">
+        <is>
+          <t>JP</t>
+        </is>
+      </c>
+      <c r="H915" s="3" t="inlineStr">
+        <is>
+          <t>Japanese</t>
+        </is>
+      </c>
+      <c r="I915" s="3" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="J915" s="3" t="inlineStr">
+        <is>
+          <t>https://gamewith.jp/</t>
+        </is>
+      </c>
+      <c r="K915" s="3" t="inlineStr"/>
+      <c r="L915" s="3" t="inlineStr"/>
+      <c r="M915" s="3" t="inlineStr"/>
+      <c r="N915" s="3" t="inlineStr"/>
+      <c r="O915" s="3" t="inlineStr"/>
+      <c r="P915" s="3" t="inlineStr"/>
+      <c r="Q915" s="3" t="inlineStr"/>
+      <c r="R915" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:R888"/>
+  <autoFilter ref="A1:R915"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -65280,7 +66900,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>95</t>
         </is>
       </c>
     </row>
@@ -65545,12 +67165,12 @@
       <c r="B19" s="3" t="inlineStr"/>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>People</t>
+          <t>Communities</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>95</t>
         </is>
       </c>
     </row>
@@ -65563,12 +67183,12 @@
       <c r="B20" s="3" t="inlineStr"/>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Communities</t>
+          <t>People</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>69</t>
         </is>
       </c>
     </row>
@@ -65586,7 +67206,7 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>167</t>
         </is>
       </c>
     </row>
@@ -66058,7 +67678,7 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>167</t>
         </is>
       </c>
     </row>
@@ -66626,7 +68246,7 @@
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>492</t>
+          <t>519</t>
         </is>
       </c>
     </row>
@@ -68664,7 +70284,7 @@
       </c>
       <c r="D170" s="3" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>53</t>
         </is>
       </c>
     </row>
@@ -68902,7 +70522,7 @@
       </c>
       <c r="D181" s="3" t="inlineStr">
         <is>
-          <t>391</t>
+          <t>418</t>
         </is>
       </c>
     </row>
@@ -69158,7 +70778,7 @@
       </c>
       <c r="D195" s="3" t="inlineStr">
         <is>
-          <t>887</t>
+          <t>914</t>
         </is>
       </c>
     </row>
@@ -69180,7 +70800,7 @@
       </c>
       <c r="D196" s="3" t="inlineStr">
         <is>
-          <t>887</t>
+          <t>914</t>
         </is>
       </c>
     </row>
@@ -69202,7 +70822,7 @@
       </c>
       <c r="D197" s="3" t="inlineStr">
         <is>
-          <t>887</t>
+          <t>914</t>
         </is>
       </c>
     </row>
@@ -69224,7 +70844,7 @@
       </c>
       <c r="D198" s="3" t="inlineStr">
         <is>
-          <t>887</t>
+          <t>914</t>
         </is>
       </c>
     </row>
@@ -69246,7 +70866,7 @@
       </c>
       <c r="D199" s="3" t="inlineStr">
         <is>
-          <t>887</t>
+          <t>914</t>
         </is>
       </c>
     </row>
@@ -69268,7 +70888,7 @@
       </c>
       <c r="D200" s="3" t="inlineStr">
         <is>
-          <t>887</t>
+          <t>914</t>
         </is>
       </c>
     </row>
@@ -69290,7 +70910,7 @@
       </c>
       <c r="D201" s="3" t="inlineStr">
         <is>
-          <t>887</t>
+          <t>914</t>
         </is>
       </c>
     </row>
@@ -69312,7 +70932,7 @@
       </c>
       <c r="D202" s="3" t="inlineStr">
         <is>
-          <t>887</t>
+          <t>914</t>
         </is>
       </c>
     </row>
@@ -69334,7 +70954,7 @@
       </c>
       <c r="D203" s="3" t="inlineStr">
         <is>
-          <t>497</t>
+          <t>524</t>
         </is>
       </c>
     </row>
@@ -69356,7 +70976,7 @@
       </c>
       <c r="D204" s="3" t="inlineStr">
         <is>
-          <t>887</t>
+          <t>914</t>
         </is>
       </c>
     </row>

</xml_diff>